<commit_message>
更新日报: 2026/08/27 周四 19:45:29.78
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\软通文件\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B98B6CA2-F978-45C1-B793-98D1034DADFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{394A3A8A-7FBD-4FC6-A577-5780EB04B8AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -539,7 +539,7 @@
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
-    <t>学习租户不在使用后 如何进行资源释放以及资源释放的规则</t>
+    <t>学习租户不在使用后 如何进行资源释放以及资源释放的规则等</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
 </sst>
@@ -1267,50 +1267,76 @@
     <xf numFmtId="0" fontId="15" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="8" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1342,75 +1368,49 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="8" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="10" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="10" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="10" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2230,178 +2230,178 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.75">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="68" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="28"/>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="70"/>
     </row>
     <row r="2" spans="1:11" ht="35" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="59" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="29"/>
+      <c r="C2" s="59"/>
       <c r="D2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="29" t="s">
+      <c r="E2" s="59" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="29"/>
+      <c r="F2" s="59"/>
       <c r="G2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="29" t="s">
+      <c r="H2" s="59" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="29"/>
-      <c r="J2" s="30"/>
+      <c r="I2" s="59"/>
+      <c r="J2" s="71"/>
       <c r="K2" s="10"/>
     </row>
     <row r="3" spans="1:11" ht="15.75">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="29" t="s">
+      <c r="B3" s="59" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="29"/>
+      <c r="C3" s="59"/>
       <c r="D3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="29" t="s">
+      <c r="E3" s="59" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="29"/>
+      <c r="F3" s="59"/>
       <c r="G3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="29" t="s">
+      <c r="H3" s="59" t="s">
         <v>14</v>
       </c>
-      <c r="I3" s="29"/>
-      <c r="J3" s="31"/>
+      <c r="I3" s="59"/>
+      <c r="J3" s="72"/>
     </row>
     <row r="4" spans="1:11" ht="15.75">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="29" t="s">
+      <c r="B4" s="59" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="29"/>
-      <c r="D4" s="29"/>
-      <c r="E4" s="29"/>
-      <c r="F4" s="32" t="s">
+      <c r="C4" s="59"/>
+      <c r="D4" s="59"/>
+      <c r="E4" s="59"/>
+      <c r="F4" s="60" t="s">
         <v>17</v>
       </c>
-      <c r="G4" s="32"/>
-      <c r="H4" s="33" t="s">
+      <c r="G4" s="60"/>
+      <c r="H4" s="61" t="s">
         <v>18</v>
       </c>
-      <c r="I4" s="34"/>
-      <c r="J4" s="35"/>
+      <c r="I4" s="62"/>
+      <c r="J4" s="63"/>
     </row>
     <row r="5" spans="1:11" ht="15.75">
-      <c r="A5" s="36" t="s">
+      <c r="A5" s="64" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="32"/>
-      <c r="C5" s="32"/>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32"/>
-      <c r="F5" s="29" t="s">
+      <c r="B5" s="60"/>
+      <c r="C5" s="60"/>
+      <c r="D5" s="60"/>
+      <c r="E5" s="60"/>
+      <c r="F5" s="59" t="s">
         <v>20</v>
       </c>
-      <c r="G5" s="29"/>
-      <c r="H5" s="37" t="s">
+      <c r="G5" s="59"/>
+      <c r="H5" s="65" t="s">
         <v>21</v>
       </c>
-      <c r="I5" s="38"/>
-      <c r="J5" s="39"/>
+      <c r="I5" s="66"/>
+      <c r="J5" s="67"/>
     </row>
     <row r="6" spans="1:11" ht="20.25">
-      <c r="A6" s="40" t="s">
+      <c r="A6" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="41"/>
-      <c r="C6" s="41"/>
-      <c r="D6" s="41"/>
-      <c r="E6" s="41"/>
-      <c r="F6" s="41"/>
-      <c r="G6" s="41"/>
-      <c r="H6" s="41"/>
-      <c r="I6" s="41"/>
-      <c r="J6" s="42"/>
+      <c r="B6" s="50"/>
+      <c r="C6" s="50"/>
+      <c r="D6" s="50"/>
+      <c r="E6" s="50"/>
+      <c r="F6" s="50"/>
+      <c r="G6" s="50"/>
+      <c r="H6" s="50"/>
+      <c r="I6" s="50"/>
+      <c r="J6" s="51"/>
     </row>
     <row r="7" spans="1:11" ht="353" customHeight="1">
-      <c r="A7" s="43" t="s">
+      <c r="A7" s="52" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="44"/>
-      <c r="C7" s="44"/>
-      <c r="D7" s="44"/>
-      <c r="E7" s="44"/>
-      <c r="F7" s="44"/>
-      <c r="G7" s="44"/>
-      <c r="H7" s="44"/>
-      <c r="I7" s="44"/>
-      <c r="J7" s="45"/>
+      <c r="B7" s="53"/>
+      <c r="C7" s="53"/>
+      <c r="D7" s="53"/>
+      <c r="E7" s="53"/>
+      <c r="F7" s="53"/>
+      <c r="G7" s="53"/>
+      <c r="H7" s="53"/>
+      <c r="I7" s="53"/>
+      <c r="J7" s="54"/>
       <c r="K7" s="11" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="20.25">
-      <c r="A8" s="46" t="s">
+      <c r="A8" s="55" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="47"/>
-      <c r="C8" s="47"/>
-      <c r="D8" s="47"/>
-      <c r="E8" s="47"/>
-      <c r="F8" s="47"/>
-      <c r="G8" s="47"/>
-      <c r="H8" s="47"/>
-      <c r="I8" s="47"/>
-      <c r="J8" s="48"/>
+      <c r="B8" s="56"/>
+      <c r="C8" s="56"/>
+      <c r="D8" s="56"/>
+      <c r="E8" s="56"/>
+      <c r="F8" s="56"/>
+      <c r="G8" s="56"/>
+      <c r="H8" s="56"/>
+      <c r="I8" s="56"/>
+      <c r="J8" s="57"/>
     </row>
     <row r="9" spans="1:11" ht="32" customHeight="1">
-      <c r="A9" s="49" t="s">
+      <c r="A9" s="58" t="s">
         <v>26</v>
       </c>
-      <c r="B9" s="44"/>
-      <c r="C9" s="44"/>
-      <c r="D9" s="44"/>
-      <c r="E9" s="44"/>
-      <c r="F9" s="44"/>
-      <c r="G9" s="44"/>
-      <c r="H9" s="44"/>
-      <c r="I9" s="44"/>
-      <c r="J9" s="45"/>
+      <c r="B9" s="53"/>
+      <c r="C9" s="53"/>
+      <c r="D9" s="53"/>
+      <c r="E9" s="53"/>
+      <c r="F9" s="53"/>
+      <c r="G9" s="53"/>
+      <c r="H9" s="53"/>
+      <c r="I9" s="53"/>
+      <c r="J9" s="54"/>
     </row>
     <row r="10" spans="1:11" ht="20.25">
-      <c r="A10" s="46" t="s">
+      <c r="A10" s="55" t="s">
         <v>27</v>
       </c>
-      <c r="B10" s="47"/>
-      <c r="C10" s="47"/>
-      <c r="D10" s="47"/>
-      <c r="E10" s="47"/>
-      <c r="F10" s="47"/>
-      <c r="G10" s="47"/>
-      <c r="H10" s="47"/>
-      <c r="I10" s="47"/>
-      <c r="J10" s="48"/>
+      <c r="B10" s="56"/>
+      <c r="C10" s="56"/>
+      <c r="D10" s="56"/>
+      <c r="E10" s="56"/>
+      <c r="F10" s="56"/>
+      <c r="G10" s="56"/>
+      <c r="H10" s="56"/>
+      <c r="I10" s="56"/>
+      <c r="J10" s="57"/>
     </row>
     <row r="11" spans="1:11" ht="29.25">
       <c r="A11" s="3" t="s">
@@ -2410,17 +2410,17 @@
       <c r="B11" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C11" s="50" t="s">
+      <c r="C11" s="41" t="s">
         <v>30</v>
       </c>
-      <c r="D11" s="51"/>
+      <c r="D11" s="42"/>
       <c r="E11" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F11" s="52" t="s">
+      <c r="F11" s="29" t="s">
         <v>32</v>
       </c>
-      <c r="G11" s="53"/>
+      <c r="G11" s="31"/>
       <c r="H11" s="5" t="s">
         <v>33</v>
       </c>
@@ -2438,15 +2438,15 @@
       <c r="B12" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C12" s="54" t="s">
+      <c r="C12" s="43" t="s">
         <v>37</v>
       </c>
-      <c r="D12" s="55"/>
+      <c r="D12" s="44"/>
       <c r="E12" s="8"/>
-      <c r="F12" s="56" t="s">
+      <c r="F12" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="G12" s="57"/>
+      <c r="G12" s="45"/>
       <c r="H12" s="9" t="s">
         <v>36</v>
       </c>
@@ -2456,87 +2456,65 @@
       </c>
     </row>
     <row r="13" spans="1:11" ht="14" customHeight="1">
-      <c r="A13" s="58" t="s">
+      <c r="A13" s="46" t="s">
         <v>38</v>
       </c>
-      <c r="B13" s="59"/>
-      <c r="C13" s="59"/>
-      <c r="D13" s="59"/>
-      <c r="E13" s="59"/>
-      <c r="F13" s="59"/>
-      <c r="G13" s="59"/>
-      <c r="H13" s="59"/>
-      <c r="I13" s="59"/>
-      <c r="J13" s="60"/>
+      <c r="B13" s="47"/>
+      <c r="C13" s="47"/>
+      <c r="D13" s="47"/>
+      <c r="E13" s="47"/>
+      <c r="F13" s="47"/>
+      <c r="G13" s="47"/>
+      <c r="H13" s="47"/>
+      <c r="I13" s="47"/>
+      <c r="J13" s="48"/>
     </row>
     <row r="14" spans="1:11" ht="14" customHeight="1">
       <c r="A14" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B14" s="61" t="s">
+      <c r="B14" s="26" t="s">
         <v>39</v>
       </c>
-      <c r="C14" s="62"/>
-      <c r="D14" s="63"/>
-      <c r="E14" s="52" t="s">
+      <c r="C14" s="27"/>
+      <c r="D14" s="28"/>
+      <c r="E14" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="F14" s="64"/>
-      <c r="G14" s="53"/>
+      <c r="F14" s="30"/>
+      <c r="G14" s="31"/>
       <c r="H14" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="I14" s="52" t="s">
+      <c r="I14" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="J14" s="65"/>
+      <c r="J14" s="32"/>
     </row>
     <row r="15" spans="1:11" ht="14" customHeight="1">
       <c r="A15" s="6">
         <v>1</v>
       </c>
-      <c r="B15" s="66" t="s">
+      <c r="B15" s="33" t="s">
         <v>43</v>
       </c>
-      <c r="C15" s="67"/>
-      <c r="D15" s="68"/>
-      <c r="E15" s="69" t="s">
+      <c r="C15" s="34"/>
+      <c r="D15" s="35"/>
+      <c r="E15" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="F15" s="70"/>
-      <c r="G15" s="71"/>
+      <c r="F15" s="37"/>
+      <c r="G15" s="38"/>
       <c r="H15" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="I15" s="56" t="s">
+      <c r="I15" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="J15" s="72"/>
+      <c r="J15" s="40"/>
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="E14:G14"/>
-    <mergeCell ref="I14:J14"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="E15:G15"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="A13:J13"/>
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A7:J7"/>
-    <mergeCell ref="A8:J8"/>
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="A10:J10"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="H5:J5"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
@@ -2544,6 +2522,28 @@
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="E3:F3"/>
     <mergeCell ref="H3:J3"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A8:J8"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="A10:J10"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="A13:J13"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="E14:G14"/>
+    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="E15:G15"/>
+    <mergeCell ref="I15:J15"/>
   </mergeCells>
   <phoneticPr fontId="30" type="noConversion"/>
   <dataValidations count="2">

</xml_diff>

<commit_message>
更新日报: 2026/08/27 周四 20:24:56.82
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\软通文件\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{394A3A8A-7FBD-4FC6-A577-5780EB04B8AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06B96F17-E323-4D6A-B8B0-2DB4F1C36C84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1.日工作简报" sheetId="11" r:id="rId1"/>
@@ -163,41 +163,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000004000000}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <rFont val="宋体"/>
-            <family val="3"/>
-            <charset val="134"/>
-          </rPr>
-          <t xml:space="preserve">填写驻场的工程师技能及区域，如：
-</t>
-        </r>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">IT &amp; </t>
-        </r>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <rFont val="宋体"/>
-            <family val="3"/>
-            <charset val="134"/>
-          </rPr>
-          <t>中级</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B4" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000005000000}">
+    <comment ref="B3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000005000000}">
       <text>
         <r>
           <rPr>
@@ -331,7 +297,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="41">
+  <si>
+    <t>工作&amp;学习日报-8月27日</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
   <si>
     <r>
       <rPr>
@@ -356,6 +326,10 @@
     </r>
   </si>
   <si>
+    <t>学习了华为云中 租户 vdc 企业项目的概念  并且ManageOne 资源全流程流转图</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
     <r>
       <rPr>
         <b/>
@@ -379,51 +353,13 @@
     </r>
   </si>
   <si>
-    <t>xx局点华为云平台xx运维-驻场服务周报</t>
-  </si>
-  <si>
-    <t>项目名称</t>
-  </si>
-  <si>
-    <t>国网云xxxx-驻场服务</t>
-  </si>
-  <si>
-    <t>客户名称</t>
-  </si>
-  <si>
-    <t>内蒙古xxxx有限公司</t>
+    <t>学习租户不在使用后 如何进行资源释放以及资源释放的规则等</t>
+    <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
     <t>报告周期</t>
   </si>
   <si>
-    <t>2025年3月24日-2025年3月30日</t>
-  </si>
-  <si>
-    <t>合同号</t>
-  </si>
-  <si>
-    <t>1Y012324060053</t>
-  </si>
-  <si>
-    <t>代表处</t>
-  </si>
-  <si>
-    <t>内蒙古代表处</t>
-  </si>
-  <si>
-    <t>产品&amp;级别</t>
-  </si>
-  <si>
-    <t>云xx&amp;中级</t>
-  </si>
-  <si>
-    <t>合同周期</t>
-  </si>
-  <si>
-    <t>2024/11/25-2025/5/25</t>
-  </si>
-  <si>
     <t>姓名</t>
   </si>
   <si>
@@ -433,113 +369,127 @@
     <t>交付工程师信息</t>
   </si>
   <si>
-    <t>陈xx</t>
-  </si>
-  <si>
-    <t>177xxxxxxxx</t>
+    <t>下周工作计划</t>
+  </si>
+  <si>
+    <t>项目风险问题</t>
+  </si>
+  <si>
+    <t>序号</t>
+  </si>
+  <si>
+    <t>产生日期</t>
+  </si>
+  <si>
+    <t>问题描述&amp;影响</t>
+  </si>
+  <si>
+    <t>紧急程度</t>
+  </si>
+  <si>
+    <t>规避措施、解决进展</t>
+  </si>
+  <si>
+    <t>责任人</t>
+  </si>
+  <si>
+    <t>状态</t>
+  </si>
+  <si>
+    <t>实际关闭日期</t>
+  </si>
+  <si>
+    <t>/</t>
+  </si>
+  <si>
+    <t>求助</t>
+  </si>
+  <si>
+    <t>求助事宜</t>
+  </si>
+  <si>
+    <t>求助人</t>
+  </si>
+  <si>
+    <t>要求解决时间</t>
+  </si>
+  <si>
+    <t>备注</t>
+  </si>
+  <si>
+    <t>项目日报要求不变，参考</t>
+  </si>
+  <si>
+    <t>/</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
+    <t>能力提升-学习周报</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
+    <t>当前产品&amp;级别</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
+    <t>目标产品&amp;级别</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
+    <t>计划周期</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
+    <t>20周</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
+    <t>苏文强</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
+    <t>16611601206</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
+    <t>云计算&amp;中级</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
+    <t>云计算&amp;高级</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
+    <t>将每日日报内容直接粘贴到周报内对应日期下即可</t>
+    <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
     <t>本周工作内容</t>
-  </si>
-  <si>
-    <t>周一
-1.国网xx电力-用电需求分析数据应用体系工单问题处理。
-2.国网xx电力-HCS-告警处理。
-3.国网xx电力-HCS-DCS3.0从节点规避漏洞后启动失败问题排查处理。
-周二
-1.国网xx电力-用电需求分析数据应用体系工单问题处理。
-2.国网xx电力-HCS-告警处理。
-3.国网xx电力-HCS-DCS3.0从节点规避漏洞后启动失败问题排查处理。
-周三
-1.国网xx电力-用电需求分析数据应用体系工单问题处理。
-2.国网xx电力-HCS-告警处理。
-3.国网xx电力-HCS-DCS3.0从节点规避漏洞后启动失败问题排查处理。
-周四
-1.国网xx电力-用电需求分析数据应用体系工单问题处理。
-2.国网xx电力-HCS-告警处理。
-3.国网xx电力-HCS-DCS3.0从节点规避漏洞后启动失败问题排查处理。
-周五
-1.国网xx电力-用电需求分析数据应用体系工单问题处理。
-2.国网xx电力-HCS-告警处理。
-3.国网xx电力-HCS-DCS3.0从节点规避漏洞后启动失败问题排查处理。
-周六
-xxxxx
-周日
-xxxxx</t>
-  </si>
-  <si>
-    <t>将每日日报内容直接粘贴到周报内对应日期下即可</t>
-  </si>
-  <si>
-    <t>下周工作计划</t>
-  </si>
-  <si>
-    <t>协助HCS产品日常维护;问题跟进及配合华为TAC处理故障</t>
-  </si>
-  <si>
-    <t>项目风险问题</t>
-  </si>
-  <si>
-    <t>序号</t>
-  </si>
-  <si>
-    <t>产生日期</t>
-  </si>
-  <si>
-    <t>问题描述&amp;影响</t>
-  </si>
-  <si>
-    <t>紧急程度</t>
-  </si>
-  <si>
-    <t>规避措施、解决进展</t>
-  </si>
-  <si>
-    <t>责任人</t>
-  </si>
-  <si>
-    <t>状态</t>
-  </si>
-  <si>
-    <t>实际关闭日期</t>
-  </si>
-  <si>
-    <t>/</t>
-  </si>
-  <si>
-    <t>新增内容再新增一行,没有填写"/"</t>
-  </si>
-  <si>
-    <t>求助</t>
-  </si>
-  <si>
-    <t>求助事宜</t>
-  </si>
-  <si>
-    <t>求助人</t>
-  </si>
-  <si>
-    <t>要求解决时间</t>
-  </si>
-  <si>
-    <t>备注</t>
-  </si>
-  <si>
-    <t>新增内容再新增一行，没有填写"/"</t>
-  </si>
-  <si>
-    <t>项目日报要求不变，参考</t>
-  </si>
-  <si>
-    <t>工作&amp;学习日报-8月27日</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
-    <t>学习了华为云中 租户 vdc 企业项目的概念  并且ManageOne 资源全流程流转图</t>
+    <t>学习华为私有云部署</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
-    <t>学习租户不在使用后 如何进行资源释放以及资源释放的规则等</t>
+    <t>2026年8月24日-2026年8月28日</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
+    <t>周一:
+1.学习了私有云部署的第四阶段: 导入 LLD 并一键批量部署 登录HCC Turnkey 上传LLD表格与软件包 参数预校验最后进行一键自动安装
+2; 阶段 5：自动化巡检与业务验证 主要进行健康检查 时钟同步校验 和首个业务的验证
+周二:
+1. 学习了新租户业务上线标准执行流程 一阶段: 底座资源与规格配置 进入规格管理 创建业务计算规格 关键打标（自动触发同步）
+2. 阶段二: 租户治理与路权下发 创建 VDC 组织与用户 创建资源空间（绑定物理区域） 资源池授权至下级 VDC 外部网络划拨
+周三:
+1. 学习了第三阶段 租户网络构建与虚拟机发放 首先申请业务 VPC 与子网 再创建安全组与服务器组 最后发放业务虚拟机即可 
+2. 交付过程中遇到的问题与解决方案: serviceom创建规格后 无同步按钮: 只要绑定了对应的az的主机组 就会自动同步到manage one运营面 (2) 新建租户的服务列表为空: 要以管理员身份登录运营面 进行资源空间的创建 (3)租户申请VPC时候 外部网络没有数据可以选择: 管理员账号 进入租户管理 选择网络资源-&gt;外部网络资源 将对应网段进行分配即可
+周四:
+1. 学习了华为云中租户 VDC和企业项目的概念与联系: 其中租户是最高登记的实体用户 创建租户时候 会绑定创建一个一级VDC 然后在创建二级 三级等下级VDC 一级VDC掌握这管理源分配的给他的资源 可以分配给下级VDC 最后在将不同的业务系统对应的虚拟机 划分到不同的企业项目中 实现隔离
+周五:
+1. 学习了私有云部署第二阶段 服务器与机柜施工：服务器按LLD规划的U位上架 交换机预配置 在接入交换机上配置各端口的 VLAN、Trunk/Access 属性 堆叠M-LAG等
+2. 第三阶段: 安装首节点: 选择第 1 台控制节点物理服务器作为首节点 通过笔记本连接该服务器的 BMC 网页界面 挂载 HCS Deployer 部署工具的 ISO 镜像文件 装完操作系统 配置临时ip</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
 </sst>
@@ -552,7 +502,7 @@
     <numFmt numFmtId="176" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ \¥* #,##0.00_ ;_ \¥* \-#,##0.00_ ;_ \¥* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="31">
+  <fonts count="36">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -595,13 +545,6 @@
     <font>
       <b/>
       <sz val="10"/>
-      <name val="宋体"/>
-      <family val="3"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
       <name val="微软雅黑"/>
       <family val="2"/>
       <charset val="134"/>
@@ -664,6 +607,13 @@
       <charset val="134"/>
     </font>
     <font>
+      <b/>
+      <sz val="10"/>
+      <name val="华文细黑"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <sz val="10"/>
       <name val="华文细黑"/>
       <family val="3"/>
@@ -751,11 +701,12 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="10"/>
-      <name val="华文细黑"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
       <family val="3"/>
       <charset val="134"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
@@ -763,6 +714,44 @@
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="微软雅黑"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color indexed="12"/>
+      <name val="微软雅黑"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="微软雅黑"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="微软雅黑"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="8">
@@ -1188,68 +1177,217 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="10" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="5" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1258,7 +1396,7 @@
     <xf numFmtId="0" fontId="15" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1266,152 +1404,6 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="10" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="10" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="10" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="8" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="166">
@@ -2124,74 +2116,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="22.5" customHeight="1">
-      <c r="A1" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
+      <c r="A1" s="65" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="65"/>
+      <c r="C1" s="65"/>
+      <c r="D1" s="65"/>
+      <c r="E1" s="65"/>
+      <c r="F1" s="65"/>
+      <c r="G1" s="65"/>
+      <c r="H1" s="65"/>
     </row>
     <row r="2" spans="1:8" ht="20.25" customHeight="1">
-      <c r="A2" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
+      <c r="A2" s="66" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="67"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
     </row>
     <row r="3" spans="1:8" ht="114" customHeight="1">
-      <c r="A3" s="20" t="s">
-        <v>46</v>
-      </c>
-      <c r="B3" s="21"/>
-      <c r="C3" s="21"/>
-      <c r="D3" s="21"/>
-      <c r="E3" s="21"/>
-      <c r="F3" s="21"/>
-      <c r="G3" s="21"/>
-      <c r="H3" s="22"/>
+      <c r="A3" s="68" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="69"/>
+      <c r="C3" s="69"/>
+      <c r="D3" s="69"/>
+      <c r="E3" s="69"/>
+      <c r="F3" s="69"/>
+      <c r="G3" s="69"/>
+      <c r="H3" s="70"/>
     </row>
     <row r="4" spans="1:8" ht="54.75" customHeight="1">
-      <c r="A4" s="18" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19"/>
+      <c r="A4" s="66" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="67"/>
+      <c r="C4" s="67"/>
+      <c r="D4" s="67"/>
+      <c r="E4" s="67"/>
+      <c r="F4" s="67"/>
+      <c r="G4" s="67"/>
+      <c r="H4" s="67"/>
     </row>
     <row r="5" spans="1:8" ht="90" customHeight="1">
-      <c r="A5" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="B5" s="24"/>
-      <c r="C5" s="24"/>
-      <c r="D5" s="24"/>
-      <c r="E5" s="24"/>
-      <c r="F5" s="24"/>
-      <c r="G5" s="24"/>
-      <c r="H5" s="25"/>
+      <c r="A5" s="71" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="72"/>
+      <c r="C5" s="72"/>
+      <c r="D5" s="72"/>
+      <c r="E5" s="72"/>
+      <c r="F5" s="72"/>
+      <c r="G5" s="72"/>
+      <c r="H5" s="73"/>
     </row>
     <row r="6" spans="1:8" ht="14.25" customHeight="1">
-      <c r="A6" s="14"/>
-      <c r="B6" s="15"/>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="16"/>
+      <c r="A6" s="62"/>
+      <c r="B6" s="63"/>
+      <c r="C6" s="63"/>
+      <c r="D6" s="63"/>
+      <c r="E6" s="63"/>
+      <c r="F6" s="63"/>
+      <c r="G6" s="63"/>
+      <c r="H6" s="64"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2214,7 +2206,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="8.796875" customWidth="1"/>
@@ -2230,327 +2222,300 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.75">
-      <c r="A1" s="68" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
-      <c r="J1" s="70"/>
+      <c r="A1" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="17"/>
     </row>
     <row r="2" spans="1:11" ht="35" customHeight="1">
-      <c r="A2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="59" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="59"/>
-      <c r="D2" s="2" t="s">
+      <c r="A2" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="19"/>
+      <c r="D2" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="E2" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="F2" s="19"/>
+      <c r="G2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="59" t="s">
-        <v>6</v>
-      </c>
-      <c r="F2" s="59"/>
-      <c r="G2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="H2" s="59" t="s">
-        <v>8</v>
-      </c>
-      <c r="I2" s="59"/>
-      <c r="J2" s="71"/>
-      <c r="K2" s="10"/>
+      <c r="H2" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="I2" s="19"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="9"/>
     </row>
     <row r="3" spans="1:11" ht="15.75">
-      <c r="A3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="59" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="59"/>
-      <c r="D3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="59" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="59"/>
-      <c r="G3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H3" s="59" t="s">
-        <v>14</v>
-      </c>
-      <c r="I3" s="59"/>
-      <c r="J3" s="72"/>
+      <c r="A3" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="G3" s="21"/>
+      <c r="H3" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="I3" s="23"/>
+      <c r="J3" s="24"/>
     </row>
     <row r="4" spans="1:11" ht="15.75">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="25" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="G4" s="19"/>
+      <c r="H4" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="I4" s="27"/>
+      <c r="J4" s="28"/>
+    </row>
+    <row r="5" spans="1:11" ht="20.25">
+      <c r="A5" s="29" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5" s="30"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="31"/>
+    </row>
+    <row r="6" spans="1:11" ht="353" customHeight="1">
+      <c r="A6" s="32" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="33"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="33"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="33"/>
+      <c r="I6" s="33"/>
+      <c r="J6" s="34"/>
+      <c r="K6" s="14" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="20.25">
+      <c r="A7" s="35" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="36"/>
+      <c r="C7" s="36"/>
+      <c r="D7" s="36"/>
+      <c r="E7" s="36"/>
+      <c r="F7" s="36"/>
+      <c r="G7" s="36"/>
+      <c r="H7" s="36"/>
+      <c r="I7" s="36"/>
+      <c r="J7" s="37"/>
+    </row>
+    <row r="8" spans="1:11" ht="32" customHeight="1">
+      <c r="A8" s="38" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" s="33"/>
+      <c r="C8" s="33"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="33"/>
+      <c r="F8" s="33"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="33"/>
+      <c r="I8" s="33"/>
+      <c r="J8" s="34"/>
+    </row>
+    <row r="9" spans="1:11" ht="20.25">
+      <c r="A9" s="35" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="36"/>
+      <c r="C9" s="36"/>
+      <c r="D9" s="36"/>
+      <c r="E9" s="36"/>
+      <c r="F9" s="36"/>
+      <c r="G9" s="36"/>
+      <c r="H9" s="36"/>
+      <c r="I9" s="36"/>
+      <c r="J9" s="37"/>
+    </row>
+    <row r="10" spans="1:11" ht="29.25">
+      <c r="A10" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="39" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="40"/>
+      <c r="E10" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="59" t="s">
+      <c r="G10" s="42"/>
+      <c r="H10" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="59"/>
-      <c r="D4" s="59"/>
-      <c r="E4" s="59"/>
-      <c r="F4" s="60" t="s">
+      <c r="I10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G4" s="60"/>
-      <c r="H4" s="61" t="s">
+      <c r="J10" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="I4" s="62"/>
-      <c r="J4" s="63"/>
     </row>
-    <row r="5" spans="1:11" ht="15.75">
-      <c r="A5" s="64" t="s">
+    <row r="11" spans="1:11" ht="38" customHeight="1">
+      <c r="A11" s="5">
+        <v>1</v>
+      </c>
+      <c r="B11" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="60"/>
-      <c r="C5" s="60"/>
-      <c r="D5" s="60"/>
-      <c r="E5" s="60"/>
-      <c r="F5" s="59" t="s">
+      <c r="C11" s="51" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" s="52"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="49" t="s">
+        <v>19</v>
+      </c>
+      <c r="G11" s="53"/>
+      <c r="H11" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="I11" s="8"/>
+      <c r="J11" s="11" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="14" customHeight="1">
+      <c r="A12" s="54" t="s">
         <v>20</v>
       </c>
-      <c r="G5" s="59"/>
-      <c r="H5" s="65" t="s">
-        <v>21</v>
-      </c>
-      <c r="I5" s="66"/>
-      <c r="J5" s="67"/>
-    </row>
-    <row r="6" spans="1:11" ht="20.25">
-      <c r="A6" s="49" t="s">
-        <v>22</v>
-      </c>
-      <c r="B6" s="50"/>
-      <c r="C6" s="50"/>
-      <c r="D6" s="50"/>
-      <c r="E6" s="50"/>
-      <c r="F6" s="50"/>
-      <c r="G6" s="50"/>
-      <c r="H6" s="50"/>
-      <c r="I6" s="50"/>
-      <c r="J6" s="51"/>
-    </row>
-    <row r="7" spans="1:11" ht="353" customHeight="1">
-      <c r="A7" s="52" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" s="53"/>
-      <c r="C7" s="53"/>
-      <c r="D7" s="53"/>
-      <c r="E7" s="53"/>
-      <c r="F7" s="53"/>
-      <c r="G7" s="53"/>
-      <c r="H7" s="53"/>
-      <c r="I7" s="53"/>
-      <c r="J7" s="54"/>
-      <c r="K7" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="20.25">
-      <c r="A8" s="55" t="s">
-        <v>25</v>
-      </c>
-      <c r="B8" s="56"/>
-      <c r="C8" s="56"/>
-      <c r="D8" s="56"/>
-      <c r="E8" s="56"/>
-      <c r="F8" s="56"/>
-      <c r="G8" s="56"/>
-      <c r="H8" s="56"/>
-      <c r="I8" s="56"/>
-      <c r="J8" s="57"/>
-    </row>
-    <row r="9" spans="1:11" ht="32" customHeight="1">
-      <c r="A9" s="58" t="s">
-        <v>26</v>
-      </c>
-      <c r="B9" s="53"/>
-      <c r="C9" s="53"/>
-      <c r="D9" s="53"/>
-      <c r="E9" s="53"/>
-      <c r="F9" s="53"/>
-      <c r="G9" s="53"/>
-      <c r="H9" s="53"/>
-      <c r="I9" s="53"/>
-      <c r="J9" s="54"/>
-    </row>
-    <row r="10" spans="1:11" ht="20.25">
-      <c r="A10" s="55" t="s">
-        <v>27</v>
-      </c>
-      <c r="B10" s="56"/>
-      <c r="C10" s="56"/>
-      <c r="D10" s="56"/>
-      <c r="E10" s="56"/>
-      <c r="F10" s="56"/>
-      <c r="G10" s="56"/>
-      <c r="H10" s="56"/>
-      <c r="I10" s="56"/>
-      <c r="J10" s="57"/>
-    </row>
-    <row r="11" spans="1:11" ht="29.25">
-      <c r="A11" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C11" s="41" t="s">
-        <v>30</v>
-      </c>
-      <c r="D11" s="42"/>
-      <c r="E11" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="F11" s="29" t="s">
-        <v>32</v>
-      </c>
-      <c r="G11" s="31"/>
-      <c r="H11" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I11" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="J11" s="12" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="38" customHeight="1">
-      <c r="A12" s="6">
-        <v>1</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="C12" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="D12" s="44"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="G12" s="45"/>
-      <c r="H12" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="I12" s="9"/>
-      <c r="J12" s="13" t="s">
-        <v>36</v>
-      </c>
+      <c r="B12" s="55"/>
+      <c r="C12" s="55"/>
+      <c r="D12" s="55"/>
+      <c r="E12" s="55"/>
+      <c r="F12" s="55"/>
+      <c r="G12" s="55"/>
+      <c r="H12" s="55"/>
+      <c r="I12" s="55"/>
+      <c r="J12" s="56"/>
     </row>
     <row r="13" spans="1:11" ht="14" customHeight="1">
-      <c r="A13" s="46" t="s">
-        <v>38</v>
-      </c>
-      <c r="B13" s="47"/>
-      <c r="C13" s="47"/>
-      <c r="D13" s="47"/>
-      <c r="E13" s="47"/>
-      <c r="F13" s="47"/>
-      <c r="G13" s="47"/>
-      <c r="H13" s="47"/>
-      <c r="I13" s="47"/>
-      <c r="J13" s="48"/>
+      <c r="A13" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" s="57" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13" s="58"/>
+      <c r="D13" s="59"/>
+      <c r="E13" s="41" t="s">
+        <v>22</v>
+      </c>
+      <c r="F13" s="60"/>
+      <c r="G13" s="42"/>
+      <c r="H13" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="I13" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="J13" s="61"/>
     </row>
     <row r="14" spans="1:11" ht="14" customHeight="1">
-      <c r="A14" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B14" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="C14" s="27"/>
-      <c r="D14" s="28"/>
-      <c r="E14" s="29" t="s">
-        <v>40</v>
-      </c>
-      <c r="F14" s="30"/>
-      <c r="G14" s="31"/>
-      <c r="H14" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="I14" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="J14" s="32"/>
-    </row>
-    <row r="15" spans="1:11" ht="14" customHeight="1">
-      <c r="A15" s="6">
+      <c r="A14" s="5">
         <v>1</v>
       </c>
-      <c r="B15" s="33" t="s">
-        <v>43</v>
-      </c>
-      <c r="C15" s="34"/>
-      <c r="D15" s="35"/>
-      <c r="E15" s="36" t="s">
-        <v>36</v>
-      </c>
-      <c r="F15" s="37"/>
-      <c r="G15" s="38"/>
-      <c r="H15" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="I15" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="J15" s="40"/>
+      <c r="B14" s="43" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" s="44"/>
+      <c r="D14" s="45"/>
+      <c r="E14" s="46" t="s">
+        <v>19</v>
+      </c>
+      <c r="F14" s="47"/>
+      <c r="G14" s="48"/>
+      <c r="H14" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="I14" s="49" t="s">
+        <v>19</v>
+      </c>
+      <c r="J14" s="50"/>
     </row>
   </sheetData>
-  <mergeCells count="29">
+  <mergeCells count="26">
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="E14:G14"/>
+    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="A12:J12"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="E13:G13"/>
+    <mergeCell ref="I13:J13"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A8:J8"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A6:J6"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:J2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:G3"/>
     <mergeCell ref="H3:J3"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="H5:J5"/>
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A7:J7"/>
-    <mergeCell ref="A8:J8"/>
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="A10:J10"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="A13:J13"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="E14:G14"/>
-    <mergeCell ref="I14:J14"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="E15:G15"/>
-    <mergeCell ref="I15:J15"/>
   </mergeCells>
   <phoneticPr fontId="30" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E12" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E11" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"紧急,重要,一般"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I12" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I11" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>"OPEN,CLOSE"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2570,7 +2535,7 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>44</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
更新日报: 2026/08/28 周五 12:32:37.89
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\软通文件\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06B96F17-E323-4D6A-B8B0-2DB4F1C36C84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9948C021-A3B8-43A0-932B-157D2AC9CE61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -299,10 +299,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="41">
   <si>
-    <t>工作&amp;学习日报-8月27日</t>
-    <phoneticPr fontId="30" type="noConversion"/>
-  </si>
-  <si>
     <r>
       <rPr>
         <b/>
@@ -326,10 +322,6 @@
     </r>
   </si>
   <si>
-    <t>学习了华为云中 租户 vdc 企业项目的概念  并且ManageOne 资源全流程流转图</t>
-    <phoneticPr fontId="30" type="noConversion"/>
-  </si>
-  <si>
     <r>
       <rPr>
         <b/>
@@ -353,10 +345,6 @@
     </r>
   </si>
   <si>
-    <t>学习租户不在使用后 如何进行资源释放以及资源释放的规则等</t>
-    <phoneticPr fontId="30" type="noConversion"/>
-  </si>
-  <si>
     <t>报告周期</t>
   </si>
   <si>
@@ -476,9 +464,21 @@
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
+    <t>工作&amp;学习日报-8月28日</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
+    <t>客户创建了租户后 不想使用 进行删除时 资源释放的规则以及操作过程</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
+    <t>学习裸金属服务的下发与资源释放流程</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
     <t>周一:
 1.学习了私有云部署的第四阶段: 导入 LLD 并一键批量部署 登录HCC Turnkey 上传LLD表格与软件包 参数预校验最后进行一键自动安装
-2; 阶段 5：自动化巡检与业务验证 主要进行健康检查 时钟同步校验 和首个业务的验证
+2: 阶段 5：自动化巡检与业务验证 主要进行健康检查 时钟同步校验 和首个业务的验证
 周二:
 1. 学习了新租户业务上线标准执行流程 一阶段: 底座资源与规格配置 进入规格管理 创建业务计算规格 关键打标（自动触发同步）
 2. 阶段二: 租户治理与路权下发 创建 VDC 组织与用户 创建资源空间（绑定物理区域） 资源池授权至下级 VDC 外部网络划拨
@@ -488,8 +488,7 @@
 周四:
 1. 学习了华为云中租户 VDC和企业项目的概念与联系: 其中租户是最高登记的实体用户 创建租户时候 会绑定创建一个一级VDC 然后在创建二级 三级等下级VDC 一级VDC掌握这管理源分配的给他的资源 可以分配给下级VDC 最后在将不同的业务系统对应的虚拟机 划分到不同的企业项目中 实现隔离
 周五:
-1. 学习了私有云部署第二阶段 服务器与机柜施工：服务器按LLD规划的U位上架 交换机预配置 在接入交换机上配置各端口的 VLAN、Trunk/Access 属性 堆叠M-LAG等
-2. 第三阶段: 安装首节点: 选择第 1 台控制节点物理服务器作为首节点 通过笔记本连接该服务器的 BMC 网页界面 挂载 HCS Deployer 部署工具的 ISO 镜像文件 装完操作系统 配置临时ip</t>
+1. 学习了客户释放租户过程中 资源释放的过程和规则 1. 清空计算与存储资源 2. 拆除网络拓扑和释放弹性公网ip 3. 回收路权与解绑资源池 4. 按层级注销组织实体</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
 </sst>
@@ -1223,37 +1222,105 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="5" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1280,93 +1347,25 @@
     <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="5" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2117,7 +2116,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="22.5" customHeight="1">
       <c r="A1" s="65" t="s">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="B1" s="65"/>
       <c r="C1" s="65"/>
@@ -2129,7 +2128,7 @@
     </row>
     <row r="2" spans="1:8" ht="20.25" customHeight="1">
       <c r="A2" s="66" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B2" s="67"/>
       <c r="C2" s="67"/>
@@ -2141,7 +2140,7 @@
     </row>
     <row r="3" spans="1:8" ht="114" customHeight="1">
       <c r="A3" s="68" t="s">
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="B3" s="69"/>
       <c r="C3" s="69"/>
@@ -2153,7 +2152,7 @@
     </row>
     <row r="4" spans="1:8" ht="54.75" customHeight="1">
       <c r="A4" s="66" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B4" s="67"/>
       <c r="C4" s="67"/>
@@ -2165,7 +2164,7 @@
     </row>
     <row r="5" spans="1:8" ht="90" customHeight="1">
       <c r="A5" s="71" t="s">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="B5" s="72"/>
       <c r="C5" s="72"/>
@@ -2222,181 +2221,181 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.75">
-      <c r="A1" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="17"/>
+      <c r="A1" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="57"/>
     </row>
     <row r="2" spans="1:11" ht="35" customHeight="1">
       <c r="A2" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="B2" s="18" t="s">
-        <v>34</v>
-      </c>
-      <c r="C2" s="19"/>
+        <v>25</v>
+      </c>
+      <c r="B2" s="46" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="47"/>
       <c r="D2" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="E2" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="F2" s="19"/>
+        <v>26</v>
+      </c>
+      <c r="E2" s="46" t="s">
+        <v>32</v>
+      </c>
+      <c r="F2" s="47"/>
       <c r="G2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H2" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="I2" s="19"/>
-      <c r="J2" s="20"/>
+        <v>2</v>
+      </c>
+      <c r="H2" s="47" t="s">
+        <v>36</v>
+      </c>
+      <c r="I2" s="47"/>
+      <c r="J2" s="58"/>
       <c r="K2" s="9"/>
     </row>
     <row r="3" spans="1:11" ht="15.75">
       <c r="A3" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B3" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="21" t="s">
-        <v>6</v>
-      </c>
-      <c r="G3" s="21"/>
-      <c r="H3" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3" s="23"/>
-      <c r="J3" s="24"/>
+        <v>27</v>
+      </c>
+      <c r="B3" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="G3" s="45"/>
+      <c r="H3" s="59" t="s">
+        <v>4</v>
+      </c>
+      <c r="I3" s="60"/>
+      <c r="J3" s="61"/>
     </row>
     <row r="4" spans="1:11" ht="15.75">
-      <c r="A4" s="25" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="18" t="s">
-        <v>32</v>
-      </c>
-      <c r="G4" s="19"/>
-      <c r="H4" s="26" t="s">
-        <v>33</v>
-      </c>
-      <c r="I4" s="27"/>
-      <c r="J4" s="28"/>
+      <c r="A4" s="44" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="45"/>
+      <c r="C4" s="45"/>
+      <c r="D4" s="45"/>
+      <c r="E4" s="45"/>
+      <c r="F4" s="46" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" s="47"/>
+      <c r="H4" s="48" t="s">
+        <v>30</v>
+      </c>
+      <c r="I4" s="49"/>
+      <c r="J4" s="50"/>
     </row>
     <row r="5" spans="1:11" ht="20.25">
-      <c r="A5" s="29" t="s">
-        <v>37</v>
-      </c>
-      <c r="B5" s="30"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="31"/>
+      <c r="A5" s="51" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" s="52"/>
+      <c r="C5" s="52"/>
+      <c r="D5" s="52"/>
+      <c r="E5" s="52"/>
+      <c r="F5" s="52"/>
+      <c r="G5" s="52"/>
+      <c r="H5" s="52"/>
+      <c r="I5" s="52"/>
+      <c r="J5" s="53"/>
     </row>
     <row r="6" spans="1:11" ht="353" customHeight="1">
-      <c r="A6" s="32" t="s">
+      <c r="A6" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="33"/>
-      <c r="C6" s="33"/>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
-      <c r="F6" s="33"/>
-      <c r="G6" s="33"/>
-      <c r="H6" s="33"/>
-      <c r="I6" s="33"/>
-      <c r="J6" s="34"/>
+      <c r="B6" s="40"/>
+      <c r="C6" s="40"/>
+      <c r="D6" s="40"/>
+      <c r="E6" s="40"/>
+      <c r="F6" s="40"/>
+      <c r="G6" s="40"/>
+      <c r="H6" s="40"/>
+      <c r="I6" s="40"/>
+      <c r="J6" s="41"/>
       <c r="K6" s="14" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="20.25">
-      <c r="A7" s="35" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="36"/>
-      <c r="C7" s="36"/>
-      <c r="D7" s="36"/>
-      <c r="E7" s="36"/>
-      <c r="F7" s="36"/>
-      <c r="G7" s="36"/>
-      <c r="H7" s="36"/>
-      <c r="I7" s="36"/>
-      <c r="J7" s="37"/>
+      <c r="A7" s="36" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="37"/>
+      <c r="C7" s="37"/>
+      <c r="D7" s="37"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="37"/>
+      <c r="I7" s="37"/>
+      <c r="J7" s="38"/>
     </row>
     <row r="8" spans="1:11" ht="32" customHeight="1">
-      <c r="A8" s="38" t="s">
-        <v>38</v>
-      </c>
-      <c r="B8" s="33"/>
-      <c r="C8" s="33"/>
-      <c r="D8" s="33"/>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="33"/>
-      <c r="I8" s="33"/>
-      <c r="J8" s="34"/>
+      <c r="A8" s="39" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" s="40"/>
+      <c r="C8" s="40"/>
+      <c r="D8" s="40"/>
+      <c r="E8" s="40"/>
+      <c r="F8" s="40"/>
+      <c r="G8" s="40"/>
+      <c r="H8" s="40"/>
+      <c r="I8" s="40"/>
+      <c r="J8" s="41"/>
     </row>
     <row r="9" spans="1:11" ht="20.25">
-      <c r="A9" s="35" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" s="36"/>
-      <c r="C9" s="36"/>
-      <c r="D9" s="36"/>
-      <c r="E9" s="36"/>
-      <c r="F9" s="36"/>
-      <c r="G9" s="36"/>
-      <c r="H9" s="36"/>
-      <c r="I9" s="36"/>
-      <c r="J9" s="37"/>
+      <c r="A9" s="36" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="37"/>
+      <c r="C9" s="37"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="37"/>
+      <c r="F9" s="37"/>
+      <c r="G9" s="37"/>
+      <c r="H9" s="37"/>
+      <c r="I9" s="37"/>
+      <c r="J9" s="38"/>
     </row>
     <row r="10" spans="1:11" ht="29.25">
       <c r="A10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" s="42" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="43"/>
+      <c r="E10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="F10" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="39" t="s">
+      <c r="G10" s="34"/>
+      <c r="H10" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D10" s="40"/>
-      <c r="E10" s="4" t="s">
+      <c r="I10" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F10" s="41" t="s">
+      <c r="J10" s="10" t="s">
         <v>15</v>
-      </c>
-      <c r="G10" s="42"/>
-      <c r="H10" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="J10" s="10" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="38" customHeight="1">
@@ -2404,85 +2403,102 @@
         <v>1</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11" s="51" t="s">
-        <v>26</v>
-      </c>
-      <c r="D11" s="52"/>
+        <v>16</v>
+      </c>
+      <c r="C11" s="23" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" s="24"/>
       <c r="E11" s="7"/>
-      <c r="F11" s="49" t="s">
-        <v>19</v>
-      </c>
-      <c r="G11" s="53"/>
+      <c r="F11" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="G11" s="25"/>
       <c r="H11" s="8" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="I11" s="8"/>
       <c r="J11" s="11" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="14" customHeight="1">
-      <c r="A12" s="54" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" s="55"/>
-      <c r="C12" s="55"/>
-      <c r="D12" s="55"/>
-      <c r="E12" s="55"/>
-      <c r="F12" s="55"/>
-      <c r="G12" s="55"/>
-      <c r="H12" s="55"/>
-      <c r="I12" s="55"/>
-      <c r="J12" s="56"/>
+      <c r="A12" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="27"/>
+      <c r="C12" s="27"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="27"/>
+      <c r="F12" s="27"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="27"/>
+      <c r="I12" s="27"/>
+      <c r="J12" s="28"/>
     </row>
     <row r="13" spans="1:11" ht="14" customHeight="1">
       <c r="A13" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13" s="57" t="s">
+        <v>8</v>
+      </c>
+      <c r="B13" s="29" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="30"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="32" t="s">
+        <v>19</v>
+      </c>
+      <c r="F13" s="33"/>
+      <c r="G13" s="34"/>
+      <c r="H13" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I13" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="C13" s="58"/>
-      <c r="D13" s="59"/>
-      <c r="E13" s="41" t="s">
-        <v>22</v>
-      </c>
-      <c r="F13" s="60"/>
-      <c r="G13" s="42"/>
-      <c r="H13" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="I13" s="41" t="s">
-        <v>24</v>
-      </c>
-      <c r="J13" s="61"/>
+      <c r="J13" s="35"/>
     </row>
     <row r="14" spans="1:11" ht="14" customHeight="1">
       <c r="A14" s="5">
         <v>1</v>
       </c>
-      <c r="B14" s="43" t="s">
-        <v>26</v>
-      </c>
-      <c r="C14" s="44"/>
-      <c r="D14" s="45"/>
-      <c r="E14" s="46" t="s">
-        <v>19</v>
-      </c>
-      <c r="F14" s="47"/>
-      <c r="G14" s="48"/>
+      <c r="B14" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="C14" s="16"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="F14" s="19"/>
+      <c r="G14" s="20"/>
       <c r="H14" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="I14" s="49" t="s">
-        <v>19</v>
-      </c>
-      <c r="J14" s="50"/>
+        <v>16</v>
+      </c>
+      <c r="I14" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="J14" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A8:J8"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="F10:G10"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="E14:G14"/>
     <mergeCell ref="I14:J14"/>
@@ -2492,23 +2508,6 @@
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="E13:G13"/>
     <mergeCell ref="I13:J13"/>
-    <mergeCell ref="A7:J7"/>
-    <mergeCell ref="A8:J8"/>
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="A5:J5"/>
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:J3"/>
   </mergeCells>
   <phoneticPr fontId="30" type="noConversion"/>
   <dataValidations count="2">
@@ -2535,7 +2534,7 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
更新日报: 2026/08/28 周五 15:36:46.39
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\软通文件\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9948C021-A3B8-43A0-932B-157D2AC9CE61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18A9BA45-DCFD-42BB-B18D-C6DE57DC4AB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1.日工作简报" sheetId="11" r:id="rId1"/>
@@ -464,10 +464,6 @@
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
-    <t>工作&amp;学习日报-8月28日</t>
-    <phoneticPr fontId="30" type="noConversion"/>
-  </si>
-  <si>
     <t>客户创建了租户后 不想使用 进行删除时 资源释放的规则以及操作过程</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
@@ -489,6 +485,10 @@
 1. 学习了华为云中租户 VDC和企业项目的概念与联系: 其中租户是最高登记的实体用户 创建租户时候 会绑定创建一个一级VDC 然后在创建二级 三级等下级VDC 一级VDC掌握这管理源分配的给他的资源 可以分配给下级VDC 最后在将不同的业务系统对应的虚拟机 划分到不同的企业项目中 实现隔离
 周五:
 1. 学习了客户释放租户过程中 资源释放的过程和规则 1. 清空计算与存储资源 2. 拆除网络拓扑和释放弹性公网ip 3. 回收路权与解绑资源池 4. 按层级注销组织实体</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
+    <t>工作&amp;学习日报-8月27日</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
 </sst>
@@ -1222,6 +1222,93 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1275,97 +1362,10 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2116,7 +2116,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="22.5" customHeight="1">
       <c r="A1" s="65" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B1" s="65"/>
       <c r="C1" s="65"/>
@@ -2140,7 +2140,7 @@
     </row>
     <row r="3" spans="1:8" ht="114" customHeight="1">
       <c r="A3" s="68" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B3" s="69"/>
       <c r="C3" s="69"/>
@@ -2164,7 +2164,7 @@
     </row>
     <row r="5" spans="1:8" ht="90" customHeight="1">
       <c r="A5" s="71" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B5" s="72"/>
       <c r="C5" s="72"/>
@@ -2221,154 +2221,154 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.75">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="57"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="17"/>
     </row>
     <row r="2" spans="1:11" ht="35" customHeight="1">
       <c r="A2" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="47"/>
+      <c r="C2" s="19"/>
       <c r="D2" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="E2" s="46" t="s">
+      <c r="E2" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="F2" s="47"/>
+      <c r="F2" s="19"/>
       <c r="G2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="47" t="s">
+      <c r="H2" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="I2" s="47"/>
-      <c r="J2" s="58"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="20"/>
       <c r="K2" s="9"/>
     </row>
     <row r="3" spans="1:11" ht="15.75">
       <c r="A3" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="46" t="s">
+      <c r="B3" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="47"/>
-      <c r="D3" s="47"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="45" t="s">
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="45"/>
-      <c r="H3" s="59" t="s">
+      <c r="G3" s="21"/>
+      <c r="H3" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="60"/>
-      <c r="J3" s="61"/>
+      <c r="I3" s="23"/>
+      <c r="J3" s="24"/>
     </row>
     <row r="4" spans="1:11" ht="15.75">
-      <c r="A4" s="44" t="s">
+      <c r="A4" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="45"/>
-      <c r="C4" s="45"/>
-      <c r="D4" s="45"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="46" t="s">
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="47"/>
-      <c r="H4" s="48" t="s">
+      <c r="G4" s="19"/>
+      <c r="H4" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="49"/>
-      <c r="J4" s="50"/>
+      <c r="I4" s="27"/>
+      <c r="J4" s="28"/>
     </row>
     <row r="5" spans="1:11" ht="20.25">
-      <c r="A5" s="51" t="s">
+      <c r="A5" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="52"/>
-      <c r="C5" s="52"/>
-      <c r="D5" s="52"/>
-      <c r="E5" s="52"/>
-      <c r="F5" s="52"/>
-      <c r="G5" s="52"/>
-      <c r="H5" s="52"/>
-      <c r="I5" s="52"/>
-      <c r="J5" s="53"/>
+      <c r="B5" s="30"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="31"/>
     </row>
     <row r="6" spans="1:11" ht="353" customHeight="1">
-      <c r="A6" s="54" t="s">
-        <v>40</v>
-      </c>
-      <c r="B6" s="40"/>
-      <c r="C6" s="40"/>
-      <c r="D6" s="40"/>
-      <c r="E6" s="40"/>
-      <c r="F6" s="40"/>
-      <c r="G6" s="40"/>
-      <c r="H6" s="40"/>
-      <c r="I6" s="40"/>
-      <c r="J6" s="41"/>
+      <c r="A6" s="32" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" s="33"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="33"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="33"/>
+      <c r="I6" s="33"/>
+      <c r="J6" s="34"/>
       <c r="K6" s="14" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="20.25">
-      <c r="A7" s="36" t="s">
+      <c r="A7" s="35" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="37"/>
-      <c r="C7" s="37"/>
-      <c r="D7" s="37"/>
-      <c r="E7" s="37"/>
-      <c r="F7" s="37"/>
-      <c r="G7" s="37"/>
-      <c r="H7" s="37"/>
-      <c r="I7" s="37"/>
-      <c r="J7" s="38"/>
+      <c r="B7" s="36"/>
+      <c r="C7" s="36"/>
+      <c r="D7" s="36"/>
+      <c r="E7" s="36"/>
+      <c r="F7" s="36"/>
+      <c r="G7" s="36"/>
+      <c r="H7" s="36"/>
+      <c r="I7" s="36"/>
+      <c r="J7" s="37"/>
     </row>
     <row r="8" spans="1:11" ht="32" customHeight="1">
-      <c r="A8" s="39" t="s">
+      <c r="A8" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="40"/>
-      <c r="C8" s="40"/>
-      <c r="D8" s="40"/>
-      <c r="E8" s="40"/>
-      <c r="F8" s="40"/>
-      <c r="G8" s="40"/>
-      <c r="H8" s="40"/>
-      <c r="I8" s="40"/>
-      <c r="J8" s="41"/>
+      <c r="B8" s="33"/>
+      <c r="C8" s="33"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="33"/>
+      <c r="F8" s="33"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="33"/>
+      <c r="I8" s="33"/>
+      <c r="J8" s="34"/>
     </row>
     <row r="9" spans="1:11" ht="20.25">
-      <c r="A9" s="36" t="s">
+      <c r="A9" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="37"/>
-      <c r="C9" s="37"/>
-      <c r="D9" s="37"/>
-      <c r="E9" s="37"/>
-      <c r="F9" s="37"/>
-      <c r="G9" s="37"/>
-      <c r="H9" s="37"/>
-      <c r="I9" s="37"/>
-      <c r="J9" s="38"/>
+      <c r="B9" s="36"/>
+      <c r="C9" s="36"/>
+      <c r="D9" s="36"/>
+      <c r="E9" s="36"/>
+      <c r="F9" s="36"/>
+      <c r="G9" s="36"/>
+      <c r="H9" s="36"/>
+      <c r="I9" s="36"/>
+      <c r="J9" s="37"/>
     </row>
     <row r="10" spans="1:11" ht="29.25">
       <c r="A10" s="2" t="s">
@@ -2377,17 +2377,17 @@
       <c r="B10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="42" t="s">
+      <c r="C10" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="43"/>
+      <c r="D10" s="40"/>
       <c r="E10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="32" t="s">
+      <c r="F10" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="34"/>
+      <c r="G10" s="42"/>
       <c r="H10" s="4" t="s">
         <v>13</v>
       </c>
@@ -2405,15 +2405,15 @@
       <c r="B11" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="23" t="s">
+      <c r="C11" s="51" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="24"/>
+      <c r="D11" s="52"/>
       <c r="E11" s="7"/>
-      <c r="F11" s="21" t="s">
+      <c r="F11" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="25"/>
+      <c r="G11" s="53"/>
       <c r="H11" s="8" t="s">
         <v>16</v>
       </c>
@@ -2423,82 +2423,65 @@
       </c>
     </row>
     <row r="12" spans="1:11" ht="14" customHeight="1">
-      <c r="A12" s="26" t="s">
+      <c r="A12" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="27"/>
-      <c r="C12" s="27"/>
-      <c r="D12" s="27"/>
-      <c r="E12" s="27"/>
-      <c r="F12" s="27"/>
-      <c r="G12" s="27"/>
-      <c r="H12" s="27"/>
-      <c r="I12" s="27"/>
-      <c r="J12" s="28"/>
+      <c r="B12" s="55"/>
+      <c r="C12" s="55"/>
+      <c r="D12" s="55"/>
+      <c r="E12" s="55"/>
+      <c r="F12" s="55"/>
+      <c r="G12" s="55"/>
+      <c r="H12" s="55"/>
+      <c r="I12" s="55"/>
+      <c r="J12" s="56"/>
     </row>
     <row r="13" spans="1:11" ht="14" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="29" t="s">
+      <c r="B13" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="30"/>
-      <c r="D13" s="31"/>
-      <c r="E13" s="32" t="s">
+      <c r="C13" s="58"/>
+      <c r="D13" s="59"/>
+      <c r="E13" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="33"/>
-      <c r="G13" s="34"/>
+      <c r="F13" s="60"/>
+      <c r="G13" s="42"/>
       <c r="H13" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="32" t="s">
+      <c r="I13" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="J13" s="35"/>
+      <c r="J13" s="61"/>
     </row>
     <row r="14" spans="1:11" ht="14" customHeight="1">
       <c r="A14" s="5">
         <v>1</v>
       </c>
-      <c r="B14" s="15" t="s">
+      <c r="B14" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="16"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="18" t="s">
+      <c r="C14" s="44"/>
+      <c r="D14" s="45"/>
+      <c r="E14" s="46" t="s">
         <v>16</v>
       </c>
-      <c r="F14" s="19"/>
-      <c r="G14" s="20"/>
+      <c r="F14" s="47"/>
+      <c r="G14" s="48"/>
       <c r="H14" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="I14" s="21" t="s">
+      <c r="I14" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="J14" s="22"/>
+      <c r="J14" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:J3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="A5:J5"/>
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A7:J7"/>
-    <mergeCell ref="A8:J8"/>
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="F10:G10"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="E14:G14"/>
     <mergeCell ref="I14:J14"/>
@@ -2508,6 +2491,23 @@
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="E13:G13"/>
     <mergeCell ref="I13:J13"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A8:J8"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:J3"/>
   </mergeCells>
   <phoneticPr fontId="30" type="noConversion"/>
   <dataValidations count="2">

</xml_diff>

<commit_message>
更新日报: 2026/08/28 周五 15:56:16.86
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\软通文件\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18A9BA45-DCFD-42BB-B18D-C6DE57DC4AB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFFF321E-79C6-41AB-8102-84860A4C22DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1.日工作简报" sheetId="11" r:id="rId1"/>
@@ -468,7 +468,11 @@
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
-    <t>学习裸金属服务的下发与资源释放流程</t>
+    <t>工作&amp;学习日报-8月28日</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
+    <t>学习裸金属服务的下发与资源释放流程和规则</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
@@ -484,11 +488,7 @@
 周四:
 1. 学习了华为云中租户 VDC和企业项目的概念与联系: 其中租户是最高登记的实体用户 创建租户时候 会绑定创建一个一级VDC 然后在创建二级 三级等下级VDC 一级VDC掌握这管理源分配的给他的资源 可以分配给下级VDC 最后在将不同的业务系统对应的虚拟机 划分到不同的企业项目中 实现隔离
 周五:
-1. 学习了客户释放租户过程中 资源释放的过程和规则 1. 清空计算与存储资源 2. 拆除网络拓扑和释放弹性公网ip 3. 回收路权与解绑资源池 4. 按层级注销组织实体</t>
-    <phoneticPr fontId="30" type="noConversion"/>
-  </si>
-  <si>
-    <t>工作&amp;学习日报-8月27日</t>
+1. 学习了客户释放租户过程中 资源释放的过程和规则 1. 清空计算与存储资源 2. 拆除网络拓扑和释放弹性公网ip 3. 解绑资源池并回收资源授权 4. 按层级注销组织实体</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
 </sst>
@@ -1222,37 +1222,141 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="5" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1279,130 +1383,26 @@
     <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="5" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="166">
@@ -2115,74 +2115,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="22.5" customHeight="1">
-      <c r="A1" s="65" t="s">
-        <v>40</v>
-      </c>
-      <c r="B1" s="65"/>
-      <c r="C1" s="65"/>
-      <c r="D1" s="65"/>
-      <c r="E1" s="65"/>
-      <c r="F1" s="65"/>
-      <c r="G1" s="65"/>
-      <c r="H1" s="65"/>
+      <c r="A1" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
     </row>
     <row r="2" spans="1:8" ht="20.25" customHeight="1">
-      <c r="A2" s="66" t="s">
+      <c r="A2" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="67"/>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
     </row>
     <row r="3" spans="1:8" ht="114" customHeight="1">
-      <c r="A3" s="68" t="s">
+      <c r="A3" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="B3" s="69"/>
-      <c r="C3" s="69"/>
-      <c r="D3" s="69"/>
-      <c r="E3" s="69"/>
-      <c r="F3" s="69"/>
-      <c r="G3" s="69"/>
-      <c r="H3" s="70"/>
+      <c r="B3" s="22"/>
+      <c r="C3" s="22"/>
+      <c r="D3" s="22"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="22"/>
+      <c r="G3" s="22"/>
+      <c r="H3" s="23"/>
     </row>
     <row r="4" spans="1:8" ht="54.75" customHeight="1">
-      <c r="A4" s="66" t="s">
+      <c r="A4" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="67"/>
-      <c r="C4" s="67"/>
-      <c r="D4" s="67"/>
-      <c r="E4" s="67"/>
-      <c r="F4" s="67"/>
-      <c r="G4" s="67"/>
-      <c r="H4" s="67"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="20"/>
+      <c r="H4" s="20"/>
     </row>
     <row r="5" spans="1:8" ht="90" customHeight="1">
-      <c r="A5" s="71" t="s">
-        <v>38</v>
-      </c>
-      <c r="B5" s="72"/>
-      <c r="C5" s="72"/>
-      <c r="D5" s="72"/>
-      <c r="E5" s="72"/>
-      <c r="F5" s="72"/>
-      <c r="G5" s="72"/>
-      <c r="H5" s="73"/>
+      <c r="A5" s="24" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="25"/>
+      <c r="C5" s="25"/>
+      <c r="D5" s="25"/>
+      <c r="E5" s="25"/>
+      <c r="F5" s="25"/>
+      <c r="G5" s="25"/>
+      <c r="H5" s="26"/>
     </row>
     <row r="6" spans="1:8" ht="14.25" customHeight="1">
-      <c r="A6" s="62"/>
-      <c r="B6" s="63"/>
-      <c r="C6" s="63"/>
-      <c r="D6" s="63"/>
-      <c r="E6" s="63"/>
-      <c r="F6" s="63"/>
-      <c r="G6" s="63"/>
-      <c r="H6" s="64"/>
+      <c r="A6" s="15"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2221,154 +2221,154 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.75">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="17"/>
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
+      <c r="D1" s="68"/>
+      <c r="E1" s="68"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="68"/>
+      <c r="H1" s="68"/>
+      <c r="I1" s="68"/>
+      <c r="J1" s="69"/>
     </row>
     <row r="2" spans="1:11" ht="35" customHeight="1">
       <c r="A2" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="58" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="19"/>
+      <c r="C2" s="59"/>
       <c r="D2" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="58" t="s">
         <v>32</v>
       </c>
-      <c r="F2" s="19"/>
+      <c r="F2" s="59"/>
       <c r="G2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="19" t="s">
+      <c r="H2" s="59" t="s">
         <v>36</v>
       </c>
-      <c r="I2" s="19"/>
-      <c r="J2" s="20"/>
+      <c r="I2" s="59"/>
+      <c r="J2" s="70"/>
       <c r="K2" s="9"/>
     </row>
     <row r="3" spans="1:11" ht="15.75">
       <c r="A3" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="58" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="21" t="s">
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="57" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="21"/>
-      <c r="H3" s="22" t="s">
+      <c r="G3" s="57"/>
+      <c r="H3" s="71" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="23"/>
-      <c r="J3" s="24"/>
+      <c r="I3" s="72"/>
+      <c r="J3" s="73"/>
     </row>
     <row r="4" spans="1:11" ht="15.75">
-      <c r="A4" s="25" t="s">
+      <c r="A4" s="56" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="18" t="s">
+      <c r="B4" s="57"/>
+      <c r="C4" s="57"/>
+      <c r="D4" s="57"/>
+      <c r="E4" s="57"/>
+      <c r="F4" s="58" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="19"/>
-      <c r="H4" s="26" t="s">
+      <c r="G4" s="59"/>
+      <c r="H4" s="60" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="27"/>
-      <c r="J4" s="28"/>
+      <c r="I4" s="61"/>
+      <c r="J4" s="62"/>
     </row>
     <row r="5" spans="1:11" ht="20.25">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="63" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="30"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="31"/>
+      <c r="B5" s="64"/>
+      <c r="C5" s="64"/>
+      <c r="D5" s="64"/>
+      <c r="E5" s="64"/>
+      <c r="F5" s="64"/>
+      <c r="G5" s="64"/>
+      <c r="H5" s="64"/>
+      <c r="I5" s="64"/>
+      <c r="J5" s="65"/>
     </row>
     <row r="6" spans="1:11" ht="353" customHeight="1">
-      <c r="A6" s="32" t="s">
-        <v>39</v>
-      </c>
-      <c r="B6" s="33"/>
-      <c r="C6" s="33"/>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
-      <c r="F6" s="33"/>
-      <c r="G6" s="33"/>
-      <c r="H6" s="33"/>
-      <c r="I6" s="33"/>
-      <c r="J6" s="34"/>
+      <c r="A6" s="66" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="52"/>
+      <c r="C6" s="52"/>
+      <c r="D6" s="52"/>
+      <c r="E6" s="52"/>
+      <c r="F6" s="52"/>
+      <c r="G6" s="52"/>
+      <c r="H6" s="52"/>
+      <c r="I6" s="52"/>
+      <c r="J6" s="53"/>
       <c r="K6" s="14" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="20.25">
-      <c r="A7" s="35" t="s">
+      <c r="A7" s="48" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="36"/>
-      <c r="C7" s="36"/>
-      <c r="D7" s="36"/>
-      <c r="E7" s="36"/>
-      <c r="F7" s="36"/>
-      <c r="G7" s="36"/>
-      <c r="H7" s="36"/>
-      <c r="I7" s="36"/>
-      <c r="J7" s="37"/>
+      <c r="B7" s="49"/>
+      <c r="C7" s="49"/>
+      <c r="D7" s="49"/>
+      <c r="E7" s="49"/>
+      <c r="F7" s="49"/>
+      <c r="G7" s="49"/>
+      <c r="H7" s="49"/>
+      <c r="I7" s="49"/>
+      <c r="J7" s="50"/>
     </row>
     <row r="8" spans="1:11" ht="32" customHeight="1">
-      <c r="A8" s="38" t="s">
+      <c r="A8" s="51" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="33"/>
-      <c r="C8" s="33"/>
-      <c r="D8" s="33"/>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="33"/>
-      <c r="I8" s="33"/>
-      <c r="J8" s="34"/>
+      <c r="B8" s="52"/>
+      <c r="C8" s="52"/>
+      <c r="D8" s="52"/>
+      <c r="E8" s="52"/>
+      <c r="F8" s="52"/>
+      <c r="G8" s="52"/>
+      <c r="H8" s="52"/>
+      <c r="I8" s="52"/>
+      <c r="J8" s="53"/>
     </row>
     <row r="9" spans="1:11" ht="20.25">
-      <c r="A9" s="35" t="s">
+      <c r="A9" s="48" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="36"/>
-      <c r="C9" s="36"/>
-      <c r="D9" s="36"/>
-      <c r="E9" s="36"/>
-      <c r="F9" s="36"/>
-      <c r="G9" s="36"/>
-      <c r="H9" s="36"/>
-      <c r="I9" s="36"/>
-      <c r="J9" s="37"/>
+      <c r="B9" s="49"/>
+      <c r="C9" s="49"/>
+      <c r="D9" s="49"/>
+      <c r="E9" s="49"/>
+      <c r="F9" s="49"/>
+      <c r="G9" s="49"/>
+      <c r="H9" s="49"/>
+      <c r="I9" s="49"/>
+      <c r="J9" s="50"/>
     </row>
     <row r="10" spans="1:11" ht="29.25">
       <c r="A10" s="2" t="s">
@@ -2377,17 +2377,17 @@
       <c r="B10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="39" t="s">
+      <c r="C10" s="54" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="40"/>
+      <c r="D10" s="55"/>
       <c r="E10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="41" t="s">
+      <c r="F10" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="42"/>
+      <c r="G10" s="46"/>
       <c r="H10" s="4" t="s">
         <v>13</v>
       </c>
@@ -2405,15 +2405,15 @@
       <c r="B11" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="51" t="s">
+      <c r="C11" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="52"/>
+      <c r="D11" s="36"/>
       <c r="E11" s="7"/>
-      <c r="F11" s="49" t="s">
+      <c r="F11" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="53"/>
+      <c r="G11" s="37"/>
       <c r="H11" s="8" t="s">
         <v>16</v>
       </c>
@@ -2423,65 +2423,82 @@
       </c>
     </row>
     <row r="12" spans="1:11" ht="14" customHeight="1">
-      <c r="A12" s="54" t="s">
+      <c r="A12" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="55"/>
-      <c r="C12" s="55"/>
-      <c r="D12" s="55"/>
-      <c r="E12" s="55"/>
-      <c r="F12" s="55"/>
-      <c r="G12" s="55"/>
-      <c r="H12" s="55"/>
-      <c r="I12" s="55"/>
-      <c r="J12" s="56"/>
+      <c r="B12" s="39"/>
+      <c r="C12" s="39"/>
+      <c r="D12" s="39"/>
+      <c r="E12" s="39"/>
+      <c r="F12" s="39"/>
+      <c r="G12" s="39"/>
+      <c r="H12" s="39"/>
+      <c r="I12" s="39"/>
+      <c r="J12" s="40"/>
     </row>
     <row r="13" spans="1:11" ht="14" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="57" t="s">
+      <c r="B13" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="58"/>
-      <c r="D13" s="59"/>
-      <c r="E13" s="41" t="s">
+      <c r="C13" s="42"/>
+      <c r="D13" s="43"/>
+      <c r="E13" s="44" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="60"/>
-      <c r="G13" s="42"/>
+      <c r="F13" s="45"/>
+      <c r="G13" s="46"/>
       <c r="H13" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="41" t="s">
+      <c r="I13" s="44" t="s">
         <v>21</v>
       </c>
-      <c r="J13" s="61"/>
+      <c r="J13" s="47"/>
     </row>
     <row r="14" spans="1:11" ht="14" customHeight="1">
       <c r="A14" s="5">
         <v>1</v>
       </c>
-      <c r="B14" s="43" t="s">
+      <c r="B14" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="44"/>
-      <c r="D14" s="45"/>
-      <c r="E14" s="46" t="s">
+      <c r="C14" s="28"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="F14" s="47"/>
-      <c r="G14" s="48"/>
+      <c r="F14" s="31"/>
+      <c r="G14" s="32"/>
       <c r="H14" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="I14" s="49" t="s">
+      <c r="I14" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="J14" s="50"/>
+      <c r="J14" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A8:J8"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="F10:G10"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="E14:G14"/>
     <mergeCell ref="I14:J14"/>
@@ -2491,23 +2508,6 @@
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="E13:G13"/>
     <mergeCell ref="I13:J13"/>
-    <mergeCell ref="A7:J7"/>
-    <mergeCell ref="A8:J8"/>
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="A5:J5"/>
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:J3"/>
   </mergeCells>
   <phoneticPr fontId="30" type="noConversion"/>
   <dataValidations count="2">

</xml_diff>

<commit_message>
更新日报: 2026/08/31 周一 18:57:07.63
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\软通文件\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFFF321E-79C6-41AB-8102-84860A4C22DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A251B8E1-06AF-4958-9631-18C25E88D8CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1.日工作简报" sheetId="11" r:id="rId1"/>
@@ -464,18 +464,6 @@
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
-    <t>客户创建了租户后 不想使用 进行删除时 资源释放的规则以及操作过程</t>
-    <phoneticPr fontId="30" type="noConversion"/>
-  </si>
-  <si>
-    <t>工作&amp;学习日报-8月28日</t>
-    <phoneticPr fontId="30" type="noConversion"/>
-  </si>
-  <si>
-    <t>学习裸金属服务的下发与资源释放流程和规则</t>
-    <phoneticPr fontId="30" type="noConversion"/>
-  </si>
-  <si>
     <t>周一:
 1.学习了私有云部署的第四阶段: 导入 LLD 并一键批量部署 登录HCC Turnkey 上传LLD表格与软件包 参数预校验最后进行一键自动安装
 2: 阶段 5：自动化巡检与业务验证 主要进行健康检查 时钟同步校验 和首个业务的验证
@@ -489,6 +477,18 @@
 1. 学习了华为云中租户 VDC和企业项目的概念与联系: 其中租户是最高登记的实体用户 创建租户时候 会绑定创建一个一级VDC 然后在创建二级 三级等下级VDC 一级VDC掌握这管理源分配的给他的资源 可以分配给下级VDC 最后在将不同的业务系统对应的虚拟机 划分到不同的企业项目中 实现隔离
 周五:
 1. 学习了客户释放租户过程中 资源释放的过程和规则 1. 清空计算与存储资源 2. 拆除网络拓扑和释放弹性公网ip 3. 解绑资源池并回收资源授权 4. 按层级注销组织实体</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
+    <t>工作&amp;学习日报-8月31日</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
+    <t>学习了DGC这个产品的基本功能以及产品文档中的迁移相关章节 学习了一个使用案例</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
+    <t>继续学习GDC数据迁移更高阶的用法</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
 </sst>
@@ -1222,6 +1222,152 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="5" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1257,152 +1403,6 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="5" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="166">
@@ -2115,74 +2115,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="22.5" customHeight="1">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="65" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
+      <c r="B1" s="65"/>
+      <c r="C1" s="65"/>
+      <c r="D1" s="65"/>
+      <c r="E1" s="65"/>
+      <c r="F1" s="65"/>
+      <c r="G1" s="65"/>
+      <c r="H1" s="65"/>
     </row>
     <row r="2" spans="1:8" ht="20.25" customHeight="1">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="66" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
+      <c r="B2" s="67"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
     </row>
     <row r="3" spans="1:8" ht="114" customHeight="1">
-      <c r="A3" s="21" t="s">
-        <v>37</v>
-      </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="23"/>
+      <c r="A3" s="68" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" s="69"/>
+      <c r="C3" s="69"/>
+      <c r="D3" s="69"/>
+      <c r="E3" s="69"/>
+      <c r="F3" s="69"/>
+      <c r="G3" s="69"/>
+      <c r="H3" s="70"/>
     </row>
     <row r="4" spans="1:8" ht="54.75" customHeight="1">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="66" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="20"/>
-      <c r="H4" s="20"/>
+      <c r="B4" s="67"/>
+      <c r="C4" s="67"/>
+      <c r="D4" s="67"/>
+      <c r="E4" s="67"/>
+      <c r="F4" s="67"/>
+      <c r="G4" s="67"/>
+      <c r="H4" s="67"/>
     </row>
     <row r="5" spans="1:8" ht="90" customHeight="1">
-      <c r="A5" s="24" t="s">
-        <v>39</v>
-      </c>
-      <c r="B5" s="25"/>
-      <c r="C5" s="25"/>
-      <c r="D5" s="25"/>
-      <c r="E5" s="25"/>
-      <c r="F5" s="25"/>
-      <c r="G5" s="25"/>
-      <c r="H5" s="26"/>
+      <c r="A5" s="71" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5" s="72"/>
+      <c r="C5" s="72"/>
+      <c r="D5" s="72"/>
+      <c r="E5" s="72"/>
+      <c r="F5" s="72"/>
+      <c r="G5" s="72"/>
+      <c r="H5" s="73"/>
     </row>
     <row r="6" spans="1:8" ht="14.25" customHeight="1">
-      <c r="A6" s="15"/>
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="16"/>
-      <c r="H6" s="17"/>
+      <c r="A6" s="62"/>
+      <c r="B6" s="63"/>
+      <c r="C6" s="63"/>
+      <c r="D6" s="63"/>
+      <c r="E6" s="63"/>
+      <c r="F6" s="63"/>
+      <c r="G6" s="63"/>
+      <c r="H6" s="64"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2221,154 +2221,154 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.75">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="68"/>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
-      <c r="F1" s="68"/>
-      <c r="G1" s="68"/>
-      <c r="H1" s="68"/>
-      <c r="I1" s="68"/>
-      <c r="J1" s="69"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="17"/>
     </row>
     <row r="2" spans="1:11" ht="35" customHeight="1">
       <c r="A2" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="58" t="s">
+      <c r="B2" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="59"/>
+      <c r="C2" s="19"/>
       <c r="D2" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="E2" s="58" t="s">
+      <c r="E2" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="F2" s="59"/>
+      <c r="F2" s="19"/>
       <c r="G2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="59" t="s">
+      <c r="H2" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="I2" s="59"/>
-      <c r="J2" s="70"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="20"/>
       <c r="K2" s="9"/>
     </row>
     <row r="3" spans="1:11" ht="15.75">
       <c r="A3" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="58" t="s">
+      <c r="B3" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="57" t="s">
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="57"/>
-      <c r="H3" s="71" t="s">
+      <c r="G3" s="21"/>
+      <c r="H3" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="72"/>
-      <c r="J3" s="73"/>
+      <c r="I3" s="23"/>
+      <c r="J3" s="24"/>
     </row>
     <row r="4" spans="1:11" ht="15.75">
-      <c r="A4" s="56" t="s">
+      <c r="A4" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="57"/>
-      <c r="C4" s="57"/>
-      <c r="D4" s="57"/>
-      <c r="E4" s="57"/>
-      <c r="F4" s="58" t="s">
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="59"/>
-      <c r="H4" s="60" t="s">
+      <c r="G4" s="19"/>
+      <c r="H4" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="61"/>
-      <c r="J4" s="62"/>
+      <c r="I4" s="27"/>
+      <c r="J4" s="28"/>
     </row>
     <row r="5" spans="1:11" ht="20.25">
-      <c r="A5" s="63" t="s">
+      <c r="A5" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="64"/>
-      <c r="C5" s="64"/>
-      <c r="D5" s="64"/>
-      <c r="E5" s="64"/>
-      <c r="F5" s="64"/>
-      <c r="G5" s="64"/>
-      <c r="H5" s="64"/>
-      <c r="I5" s="64"/>
-      <c r="J5" s="65"/>
+      <c r="B5" s="30"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="31"/>
     </row>
     <row r="6" spans="1:11" ht="353" customHeight="1">
-      <c r="A6" s="66" t="s">
-        <v>40</v>
-      </c>
-      <c r="B6" s="52"/>
-      <c r="C6" s="52"/>
-      <c r="D6" s="52"/>
-      <c r="E6" s="52"/>
-      <c r="F6" s="52"/>
-      <c r="G6" s="52"/>
-      <c r="H6" s="52"/>
-      <c r="I6" s="52"/>
-      <c r="J6" s="53"/>
+      <c r="A6" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="33"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="33"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="33"/>
+      <c r="I6" s="33"/>
+      <c r="J6" s="34"/>
       <c r="K6" s="14" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="20.25">
-      <c r="A7" s="48" t="s">
+      <c r="A7" s="35" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="49"/>
-      <c r="C7" s="49"/>
-      <c r="D7" s="49"/>
-      <c r="E7" s="49"/>
-      <c r="F7" s="49"/>
-      <c r="G7" s="49"/>
-      <c r="H7" s="49"/>
-      <c r="I7" s="49"/>
-      <c r="J7" s="50"/>
+      <c r="B7" s="36"/>
+      <c r="C7" s="36"/>
+      <c r="D7" s="36"/>
+      <c r="E7" s="36"/>
+      <c r="F7" s="36"/>
+      <c r="G7" s="36"/>
+      <c r="H7" s="36"/>
+      <c r="I7" s="36"/>
+      <c r="J7" s="37"/>
     </row>
     <row r="8" spans="1:11" ht="32" customHeight="1">
-      <c r="A8" s="51" t="s">
+      <c r="A8" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="52"/>
-      <c r="C8" s="52"/>
-      <c r="D8" s="52"/>
-      <c r="E8" s="52"/>
-      <c r="F8" s="52"/>
-      <c r="G8" s="52"/>
-      <c r="H8" s="52"/>
-      <c r="I8" s="52"/>
-      <c r="J8" s="53"/>
+      <c r="B8" s="33"/>
+      <c r="C8" s="33"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="33"/>
+      <c r="F8" s="33"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="33"/>
+      <c r="I8" s="33"/>
+      <c r="J8" s="34"/>
     </row>
     <row r="9" spans="1:11" ht="20.25">
-      <c r="A9" s="48" t="s">
+      <c r="A9" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="49"/>
-      <c r="C9" s="49"/>
-      <c r="D9" s="49"/>
-      <c r="E9" s="49"/>
-      <c r="F9" s="49"/>
-      <c r="G9" s="49"/>
-      <c r="H9" s="49"/>
-      <c r="I9" s="49"/>
-      <c r="J9" s="50"/>
+      <c r="B9" s="36"/>
+      <c r="C9" s="36"/>
+      <c r="D9" s="36"/>
+      <c r="E9" s="36"/>
+      <c r="F9" s="36"/>
+      <c r="G9" s="36"/>
+      <c r="H9" s="36"/>
+      <c r="I9" s="36"/>
+      <c r="J9" s="37"/>
     </row>
     <row r="10" spans="1:11" ht="29.25">
       <c r="A10" s="2" t="s">
@@ -2377,17 +2377,17 @@
       <c r="B10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="54" t="s">
+      <c r="C10" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="55"/>
+      <c r="D10" s="40"/>
       <c r="E10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="44" t="s">
+      <c r="F10" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="46"/>
+      <c r="G10" s="42"/>
       <c r="H10" s="4" t="s">
         <v>13</v>
       </c>
@@ -2405,15 +2405,15 @@
       <c r="B11" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="35" t="s">
+      <c r="C11" s="51" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="36"/>
+      <c r="D11" s="52"/>
       <c r="E11" s="7"/>
-      <c r="F11" s="33" t="s">
+      <c r="F11" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="37"/>
+      <c r="G11" s="53"/>
       <c r="H11" s="8" t="s">
         <v>16</v>
       </c>
@@ -2423,82 +2423,65 @@
       </c>
     </row>
     <row r="12" spans="1:11" ht="14" customHeight="1">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="39"/>
-      <c r="C12" s="39"/>
-      <c r="D12" s="39"/>
-      <c r="E12" s="39"/>
-      <c r="F12" s="39"/>
-      <c r="G12" s="39"/>
-      <c r="H12" s="39"/>
-      <c r="I12" s="39"/>
-      <c r="J12" s="40"/>
+      <c r="B12" s="55"/>
+      <c r="C12" s="55"/>
+      <c r="D12" s="55"/>
+      <c r="E12" s="55"/>
+      <c r="F12" s="55"/>
+      <c r="G12" s="55"/>
+      <c r="H12" s="55"/>
+      <c r="I12" s="55"/>
+      <c r="J12" s="56"/>
     </row>
     <row r="13" spans="1:11" ht="14" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="41" t="s">
+      <c r="B13" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="42"/>
-      <c r="D13" s="43"/>
-      <c r="E13" s="44" t="s">
+      <c r="C13" s="58"/>
+      <c r="D13" s="59"/>
+      <c r="E13" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="45"/>
-      <c r="G13" s="46"/>
+      <c r="F13" s="60"/>
+      <c r="G13" s="42"/>
       <c r="H13" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="44" t="s">
+      <c r="I13" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="J13" s="47"/>
+      <c r="J13" s="61"/>
     </row>
     <row r="14" spans="1:11" ht="14" customHeight="1">
       <c r="A14" s="5">
         <v>1</v>
       </c>
-      <c r="B14" s="27" t="s">
+      <c r="B14" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="28"/>
-      <c r="D14" s="29"/>
-      <c r="E14" s="30" t="s">
+      <c r="C14" s="44"/>
+      <c r="D14" s="45"/>
+      <c r="E14" s="46" t="s">
         <v>16</v>
       </c>
-      <c r="F14" s="31"/>
-      <c r="G14" s="32"/>
+      <c r="F14" s="47"/>
+      <c r="G14" s="48"/>
       <c r="H14" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="I14" s="33" t="s">
+      <c r="I14" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="J14" s="34"/>
+      <c r="J14" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:J3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="A5:J5"/>
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A7:J7"/>
-    <mergeCell ref="A8:J8"/>
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="F10:G10"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="E14:G14"/>
     <mergeCell ref="I14:J14"/>
@@ -2508,6 +2491,23 @@
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="E13:G13"/>
     <mergeCell ref="I13:J13"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A8:J8"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:J3"/>
   </mergeCells>
   <phoneticPr fontId="30" type="noConversion"/>
   <dataValidations count="2">

</xml_diff>

<commit_message>
更新日报: 2026/09/01 周二 17:34:18.16
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\软通文件\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A251B8E1-06AF-4958-9631-18C25E88D8CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1637B56E-9C82-4965-8105-B57E733214D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1.日工作简报" sheetId="11" r:id="rId1"/>
@@ -460,16 +460,27 @@
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
-    <t>2026年8月24日-2026年8月28日</t>
+    <t>2026年8月31日-2026年9月4日</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
+    <t>工作&amp;学习日报-9月1日</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
+    <t>在大唐机房做了验收指南中的租户与VDC中的创建租户 VDC 创建VDC管理员等等 还有运维管理中的资源回收站 告警处理 运维监控等测试</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
+    <t>继续做运维管理后续的测试 比如容量管理 资源拓扑 单点登录  FusionCare日常巡检等</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
     <t>周一:
-1.学习了私有云部署的第四阶段: 导入 LLD 并一键批量部署 登录HCC Turnkey 上传LLD表格与软件包 参数预校验最后进行一键自动安装
-2: 阶段 5：自动化巡检与业务验证 主要进行健康检查 时钟同步校验 和首个业务的验证
+1. 学习了GDC的基本功能 对GDC有了初步的了解 
+2. 学习GDC数据迁移的产品文档中迁移相关的章节 并且仔细学习了一个GDC数据迁移的使用案例
 周二:
-1. 学习了新租户业务上线标准执行流程 一阶段: 底座资源与规格配置 进入规格管理 创建业务计算规格 关键打标（自动触发同步）
-2. 阶段二: 租户治理与路权下发 创建 VDC 组织与用户 创建资源空间（绑定物理区域） 资源池授权至下级 VDC 外部网络划拨
+1. 在大唐机房做了验收指南中的租户与VDC中的创建租户 VDC 创建VDC管理员等等 还有运维管理中的资源回收站 告警处理 运维监控等测试
 周三:
 1. 学习了第三阶段 租户网络构建与虚拟机发放 首先申请业务 VPC 与子网 再创建安全组与服务器组 最后发放业务虚拟机即可 
 2. 交付过程中遇到的问题与解决方案: serviceom创建规格后 无同步按钮: 只要绑定了对应的az的主机组 就会自动同步到manage one运营面 (2) 新建租户的服务列表为空: 要以管理员身份登录运营面 进行资源空间的创建 (3)租户申请VPC时候 外部网络没有数据可以选择: 管理员账号 进入租户管理 选择网络资源-&gt;外部网络资源 将对应网段进行分配即可
@@ -477,18 +488,6 @@
 1. 学习了华为云中租户 VDC和企业项目的概念与联系: 其中租户是最高登记的实体用户 创建租户时候 会绑定创建一个一级VDC 然后在创建二级 三级等下级VDC 一级VDC掌握这管理源分配的给他的资源 可以分配给下级VDC 最后在将不同的业务系统对应的虚拟机 划分到不同的企业项目中 实现隔离
 周五:
 1. 学习了客户释放租户过程中 资源释放的过程和规则 1. 清空计算与存储资源 2. 拆除网络拓扑和释放弹性公网ip 3. 解绑资源池并回收资源授权 4. 按层级注销组织实体</t>
-    <phoneticPr fontId="30" type="noConversion"/>
-  </si>
-  <si>
-    <t>工作&amp;学习日报-8月31日</t>
-    <phoneticPr fontId="30" type="noConversion"/>
-  </si>
-  <si>
-    <t>学习了DGC这个产品的基本功能以及产品文档中的迁移相关章节 学习了一个使用案例</t>
-    <phoneticPr fontId="30" type="noConversion"/>
-  </si>
-  <si>
-    <t>继续学习GDC数据迁移更高阶的用法</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
 </sst>
@@ -2116,7 +2115,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="22.5" customHeight="1">
       <c r="A1" s="65" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B1" s="65"/>
       <c r="C1" s="65"/>
@@ -2140,7 +2139,7 @@
     </row>
     <row r="3" spans="1:8" ht="114" customHeight="1">
       <c r="A3" s="68" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B3" s="69"/>
       <c r="C3" s="69"/>
@@ -2164,7 +2163,7 @@
     </row>
     <row r="5" spans="1:8" ht="90" customHeight="1">
       <c r="A5" s="71" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B5" s="72"/>
       <c r="C5" s="72"/>
@@ -2313,7 +2312,7 @@
     </row>
     <row r="6" spans="1:11" ht="353" customHeight="1">
       <c r="A6" s="32" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B6" s="33"/>
       <c r="C6" s="33"/>

</xml_diff>

<commit_message>
更新日报: 2026/09/02 周三 16:50:58.00
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\软通文件\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1637B56E-9C82-4965-8105-B57E733214D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2806C995-9F75-43A9-8A60-41B2C5B5D9BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -464,15 +464,15 @@
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
-    <t>工作&amp;学习日报-9月1日</t>
+    <t>重点工作: 继续做了验收测试指南 包括单点CCAE FusionCare日常巡检 创建主门户 创建策略 以及弹性云服务器申请 注册镜像 以及各种云硬盘操作 以及对象存储服务的测试 重大风险: 无 周边求助: 无</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
-    <t>在大唐机房做了验收指南中的租户与VDC中的创建租户 VDC 创建VDC管理员等等 还有运维管理中的资源回收站 告警处理 运维监控等测试</t>
+    <t>重点工作: 依照数据治理的文档 学习数据迁移的前置操作 以及需要注意的问题</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
-    <t>继续做运维管理后续的测试 比如容量管理 资源拓扑 单点登录  FusionCare日常巡检等</t>
+    <t>工作&amp;学习日报-9月2日</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
@@ -482,8 +482,7 @@
 周二:
 1. 在大唐机房做了验收指南中的租户与VDC中的创建租户 VDC 创建VDC管理员等等 还有运维管理中的资源回收站 告警处理 运维监控等测试
 周三:
-1. 学习了第三阶段 租户网络构建与虚拟机发放 首先申请业务 VPC 与子网 再创建安全组与服务器组 最后发放业务虚拟机即可 
-2. 交付过程中遇到的问题与解决方案: serviceom创建规格后 无同步按钮: 只要绑定了对应的az的主机组 就会自动同步到manage one运营面 (2) 新建租户的服务列表为空: 要以管理员身份登录运营面 进行资源空间的创建 (3)租户申请VPC时候 外部网络没有数据可以选择: 管理员账号 进入租户管理 选择网络资源-&gt;外部网络资源 将对应网段进行分配即可
+1. 继续做了验收测试指南 包括单点CCAE FusionCare日常巡检 创建主门户 创建策略 以及弹性云服务器申请 注册镜像 以及各种云硬盘操作 以及对象存储服务的测试
 周四:
 1. 学习了华为云中租户 VDC和企业项目的概念与联系: 其中租户是最高登记的实体用户 创建租户时候 会绑定创建一个一级VDC 然后在创建二级 三级等下级VDC 一级VDC掌握这管理源分配的给他的资源 可以分配给下级VDC 最后在将不同的业务系统对应的虚拟机 划分到不同的企业项目中 实现隔离
 周五:
@@ -1221,37 +1220,105 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="5" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1278,93 +1345,25 @@
     <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="5" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2115,7 +2114,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="22.5" customHeight="1">
       <c r="A1" s="65" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B1" s="65"/>
       <c r="C1" s="65"/>
@@ -2139,7 +2138,7 @@
     </row>
     <row r="3" spans="1:8" ht="114" customHeight="1">
       <c r="A3" s="68" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B3" s="69"/>
       <c r="C3" s="69"/>
@@ -2163,7 +2162,7 @@
     </row>
     <row r="5" spans="1:8" ht="90" customHeight="1">
       <c r="A5" s="71" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B5" s="72"/>
       <c r="C5" s="72"/>
@@ -2220,154 +2219,154 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.75">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="55" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="17"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="57"/>
     </row>
     <row r="2" spans="1:11" ht="35" customHeight="1">
       <c r="A2" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="46" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="19"/>
+      <c r="C2" s="47"/>
       <c r="D2" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="46" t="s">
         <v>32</v>
       </c>
-      <c r="F2" s="19"/>
+      <c r="F2" s="47"/>
       <c r="G2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="19" t="s">
+      <c r="H2" s="47" t="s">
         <v>36</v>
       </c>
-      <c r="I2" s="19"/>
-      <c r="J2" s="20"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="58"/>
       <c r="K2" s="9"/>
     </row>
     <row r="3" spans="1:11" ht="15.75">
       <c r="A3" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="46" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="21" t="s">
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="21"/>
-      <c r="H3" s="22" t="s">
+      <c r="G3" s="45"/>
+      <c r="H3" s="59" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="23"/>
-      <c r="J3" s="24"/>
+      <c r="I3" s="60"/>
+      <c r="J3" s="61"/>
     </row>
     <row r="4" spans="1:11" ht="15.75">
-      <c r="A4" s="25" t="s">
+      <c r="A4" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="18" t="s">
+      <c r="B4" s="45"/>
+      <c r="C4" s="45"/>
+      <c r="D4" s="45"/>
+      <c r="E4" s="45"/>
+      <c r="F4" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="19"/>
-      <c r="H4" s="26" t="s">
+      <c r="G4" s="47"/>
+      <c r="H4" s="48" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="27"/>
-      <c r="J4" s="28"/>
+      <c r="I4" s="49"/>
+      <c r="J4" s="50"/>
     </row>
     <row r="5" spans="1:11" ht="20.25">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="30"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="31"/>
+      <c r="B5" s="52"/>
+      <c r="C5" s="52"/>
+      <c r="D5" s="52"/>
+      <c r="E5" s="52"/>
+      <c r="F5" s="52"/>
+      <c r="G5" s="52"/>
+      <c r="H5" s="52"/>
+      <c r="I5" s="52"/>
+      <c r="J5" s="53"/>
     </row>
     <row r="6" spans="1:11" ht="353" customHeight="1">
-      <c r="A6" s="32" t="s">
+      <c r="A6" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="33"/>
-      <c r="C6" s="33"/>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
-      <c r="F6" s="33"/>
-      <c r="G6" s="33"/>
-      <c r="H6" s="33"/>
-      <c r="I6" s="33"/>
-      <c r="J6" s="34"/>
+      <c r="B6" s="40"/>
+      <c r="C6" s="40"/>
+      <c r="D6" s="40"/>
+      <c r="E6" s="40"/>
+      <c r="F6" s="40"/>
+      <c r="G6" s="40"/>
+      <c r="H6" s="40"/>
+      <c r="I6" s="40"/>
+      <c r="J6" s="41"/>
       <c r="K6" s="14" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="20.25">
-      <c r="A7" s="35" t="s">
+      <c r="A7" s="36" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="36"/>
-      <c r="C7" s="36"/>
-      <c r="D7" s="36"/>
-      <c r="E7" s="36"/>
-      <c r="F7" s="36"/>
-      <c r="G7" s="36"/>
-      <c r="H7" s="36"/>
-      <c r="I7" s="36"/>
-      <c r="J7" s="37"/>
+      <c r="B7" s="37"/>
+      <c r="C7" s="37"/>
+      <c r="D7" s="37"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="37"/>
+      <c r="I7" s="37"/>
+      <c r="J7" s="38"/>
     </row>
     <row r="8" spans="1:11" ht="32" customHeight="1">
-      <c r="A8" s="38" t="s">
+      <c r="A8" s="39" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="33"/>
-      <c r="C8" s="33"/>
-      <c r="D8" s="33"/>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="33"/>
-      <c r="I8" s="33"/>
-      <c r="J8" s="34"/>
+      <c r="B8" s="40"/>
+      <c r="C8" s="40"/>
+      <c r="D8" s="40"/>
+      <c r="E8" s="40"/>
+      <c r="F8" s="40"/>
+      <c r="G8" s="40"/>
+      <c r="H8" s="40"/>
+      <c r="I8" s="40"/>
+      <c r="J8" s="41"/>
     </row>
     <row r="9" spans="1:11" ht="20.25">
-      <c r="A9" s="35" t="s">
+      <c r="A9" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="36"/>
-      <c r="C9" s="36"/>
-      <c r="D9" s="36"/>
-      <c r="E9" s="36"/>
-      <c r="F9" s="36"/>
-      <c r="G9" s="36"/>
-      <c r="H9" s="36"/>
-      <c r="I9" s="36"/>
-      <c r="J9" s="37"/>
+      <c r="B9" s="37"/>
+      <c r="C9" s="37"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="37"/>
+      <c r="F9" s="37"/>
+      <c r="G9" s="37"/>
+      <c r="H9" s="37"/>
+      <c r="I9" s="37"/>
+      <c r="J9" s="38"/>
     </row>
     <row r="10" spans="1:11" ht="29.25">
       <c r="A10" s="2" t="s">
@@ -2376,17 +2375,17 @@
       <c r="B10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="39" t="s">
+      <c r="C10" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="40"/>
+      <c r="D10" s="43"/>
       <c r="E10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="41" t="s">
+      <c r="F10" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="42"/>
+      <c r="G10" s="34"/>
       <c r="H10" s="4" t="s">
         <v>13</v>
       </c>
@@ -2404,15 +2403,15 @@
       <c r="B11" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="51" t="s">
+      <c r="C11" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="52"/>
+      <c r="D11" s="24"/>
       <c r="E11" s="7"/>
-      <c r="F11" s="49" t="s">
+      <c r="F11" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="53"/>
+      <c r="G11" s="25"/>
       <c r="H11" s="8" t="s">
         <v>16</v>
       </c>
@@ -2422,65 +2421,82 @@
       </c>
     </row>
     <row r="12" spans="1:11" ht="14" customHeight="1">
-      <c r="A12" s="54" t="s">
+      <c r="A12" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="55"/>
-      <c r="C12" s="55"/>
-      <c r="D12" s="55"/>
-      <c r="E12" s="55"/>
-      <c r="F12" s="55"/>
-      <c r="G12" s="55"/>
-      <c r="H12" s="55"/>
-      <c r="I12" s="55"/>
-      <c r="J12" s="56"/>
+      <c r="B12" s="27"/>
+      <c r="C12" s="27"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="27"/>
+      <c r="F12" s="27"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="27"/>
+      <c r="I12" s="27"/>
+      <c r="J12" s="28"/>
     </row>
     <row r="13" spans="1:11" ht="14" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="57" t="s">
+      <c r="B13" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="58"/>
-      <c r="D13" s="59"/>
-      <c r="E13" s="41" t="s">
+      <c r="C13" s="30"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="60"/>
-      <c r="G13" s="42"/>
+      <c r="F13" s="33"/>
+      <c r="G13" s="34"/>
       <c r="H13" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="41" t="s">
+      <c r="I13" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="J13" s="61"/>
+      <c r="J13" s="35"/>
     </row>
     <row r="14" spans="1:11" ht="14" customHeight="1">
       <c r="A14" s="5">
         <v>1</v>
       </c>
-      <c r="B14" s="43" t="s">
+      <c r="B14" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="44"/>
-      <c r="D14" s="45"/>
-      <c r="E14" s="46" t="s">
+      <c r="C14" s="16"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="F14" s="47"/>
-      <c r="G14" s="48"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="20"/>
       <c r="H14" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="I14" s="49" t="s">
+      <c r="I14" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="J14" s="50"/>
+      <c r="J14" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A8:J8"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="F10:G10"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="E14:G14"/>
     <mergeCell ref="I14:J14"/>
@@ -2490,23 +2506,6 @@
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="E13:G13"/>
     <mergeCell ref="I13:J13"/>
-    <mergeCell ref="A7:J7"/>
-    <mergeCell ref="A8:J8"/>
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="A5:J5"/>
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:J3"/>
   </mergeCells>
   <phoneticPr fontId="30" type="noConversion"/>
   <dataValidations count="2">

</xml_diff>

<commit_message>
更新日报: 2026/09/02 周三 19:54:17.00
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\软通文件\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2806C995-9F75-43A9-8A60-41B2C5B5D9BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE137767-E5FF-4459-A9CD-51867629E88C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1.日工作简报" sheetId="11" r:id="rId1"/>
@@ -464,14 +464,6 @@
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
-    <t>重点工作: 继续做了验收测试指南 包括单点CCAE FusionCare日常巡检 创建主门户 创建策略 以及弹性云服务器申请 注册镜像 以及各种云硬盘操作 以及对象存储服务的测试 重大风险: 无 周边求助: 无</t>
-    <phoneticPr fontId="30" type="noConversion"/>
-  </si>
-  <si>
-    <t>重点工作: 依照数据治理的文档 学习数据迁移的前置操作 以及需要注意的问题</t>
-    <phoneticPr fontId="30" type="noConversion"/>
-  </si>
-  <si>
     <t>工作&amp;学习日报-9月2日</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
@@ -487,6 +479,20 @@
 1. 学习了华为云中租户 VDC和企业项目的概念与联系: 其中租户是最高登记的实体用户 创建租户时候 会绑定创建一个一级VDC 然后在创建二级 三级等下级VDC 一级VDC掌握这管理源分配的给他的资源 可以分配给下级VDC 最后在将不同的业务系统对应的虚拟机 划分到不同的企业项目中 实现隔离
 周五:
 1. 学习了客户释放租户过程中 资源释放的过程和规则 1. 清空计算与存储资源 2. 拆除网络拓扑和释放弹性公网ip 3. 解绑资源池并回收资源授权 4. 按层级注销组织实体</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
+    <t>重点工作: 
+继续做了验收测试指南 包括单点CCAE FusionCare日常巡检 创建主门户 创建策略 以及弹性云服务器申请 注册镜像 以及各种云硬盘操作 以及对象存储服务的测试 
+重大风险: 无 
+周边求助: 无</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
+    <t>重点工作: 
+依照数据治理的文档 学习数据迁移的前置操作 以及需要注意的问题
+重大风险: 无 
+周边求助: 无</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
 </sst>
@@ -1220,6 +1226,93 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1273,97 +1366,10 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2114,7 +2120,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="22.5" customHeight="1">
       <c r="A1" s="65" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B1" s="65"/>
       <c r="C1" s="65"/>
@@ -2138,7 +2144,7 @@
     </row>
     <row r="3" spans="1:8" ht="114" customHeight="1">
       <c r="A3" s="68" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B3" s="69"/>
       <c r="C3" s="69"/>
@@ -2162,7 +2168,7 @@
     </row>
     <row r="5" spans="1:8" ht="90" customHeight="1">
       <c r="A5" s="71" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B5" s="72"/>
       <c r="C5" s="72"/>
@@ -2219,154 +2225,154 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.75">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="57"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="17"/>
     </row>
     <row r="2" spans="1:11" ht="35" customHeight="1">
       <c r="A2" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="47"/>
+      <c r="C2" s="19"/>
       <c r="D2" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="E2" s="46" t="s">
+      <c r="E2" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="F2" s="47"/>
+      <c r="F2" s="19"/>
       <c r="G2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="47" t="s">
+      <c r="H2" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="I2" s="47"/>
-      <c r="J2" s="58"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="20"/>
       <c r="K2" s="9"/>
     </row>
     <row r="3" spans="1:11" ht="15.75">
       <c r="A3" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="46" t="s">
+      <c r="B3" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="47"/>
-      <c r="D3" s="47"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="45" t="s">
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="45"/>
-      <c r="H3" s="59" t="s">
+      <c r="G3" s="21"/>
+      <c r="H3" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="60"/>
-      <c r="J3" s="61"/>
+      <c r="I3" s="23"/>
+      <c r="J3" s="24"/>
     </row>
     <row r="4" spans="1:11" ht="15.75">
-      <c r="A4" s="44" t="s">
+      <c r="A4" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="45"/>
-      <c r="C4" s="45"/>
-      <c r="D4" s="45"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="46" t="s">
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="47"/>
-      <c r="H4" s="48" t="s">
+      <c r="G4" s="19"/>
+      <c r="H4" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="49"/>
-      <c r="J4" s="50"/>
+      <c r="I4" s="27"/>
+      <c r="J4" s="28"/>
     </row>
     <row r="5" spans="1:11" ht="20.25">
-      <c r="A5" s="51" t="s">
+      <c r="A5" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="52"/>
-      <c r="C5" s="52"/>
-      <c r="D5" s="52"/>
-      <c r="E5" s="52"/>
-      <c r="F5" s="52"/>
-      <c r="G5" s="52"/>
-      <c r="H5" s="52"/>
-      <c r="I5" s="52"/>
-      <c r="J5" s="53"/>
+      <c r="B5" s="30"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="31"/>
     </row>
     <row r="6" spans="1:11" ht="353" customHeight="1">
-      <c r="A6" s="54" t="s">
-        <v>40</v>
-      </c>
-      <c r="B6" s="40"/>
-      <c r="C6" s="40"/>
-      <c r="D6" s="40"/>
-      <c r="E6" s="40"/>
-      <c r="F6" s="40"/>
-      <c r="G6" s="40"/>
-      <c r="H6" s="40"/>
-      <c r="I6" s="40"/>
-      <c r="J6" s="41"/>
+      <c r="A6" s="32" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="33"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="33"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="33"/>
+      <c r="I6" s="33"/>
+      <c r="J6" s="34"/>
       <c r="K6" s="14" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="20.25">
-      <c r="A7" s="36" t="s">
+      <c r="A7" s="35" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="37"/>
-      <c r="C7" s="37"/>
-      <c r="D7" s="37"/>
-      <c r="E7" s="37"/>
-      <c r="F7" s="37"/>
-      <c r="G7" s="37"/>
-      <c r="H7" s="37"/>
-      <c r="I7" s="37"/>
-      <c r="J7" s="38"/>
+      <c r="B7" s="36"/>
+      <c r="C7" s="36"/>
+      <c r="D7" s="36"/>
+      <c r="E7" s="36"/>
+      <c r="F7" s="36"/>
+      <c r="G7" s="36"/>
+      <c r="H7" s="36"/>
+      <c r="I7" s="36"/>
+      <c r="J7" s="37"/>
     </row>
     <row r="8" spans="1:11" ht="32" customHeight="1">
-      <c r="A8" s="39" t="s">
+      <c r="A8" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="40"/>
-      <c r="C8" s="40"/>
-      <c r="D8" s="40"/>
-      <c r="E8" s="40"/>
-      <c r="F8" s="40"/>
-      <c r="G8" s="40"/>
-      <c r="H8" s="40"/>
-      <c r="I8" s="40"/>
-      <c r="J8" s="41"/>
+      <c r="B8" s="33"/>
+      <c r="C8" s="33"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="33"/>
+      <c r="F8" s="33"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="33"/>
+      <c r="I8" s="33"/>
+      <c r="J8" s="34"/>
     </row>
     <row r="9" spans="1:11" ht="20.25">
-      <c r="A9" s="36" t="s">
+      <c r="A9" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="37"/>
-      <c r="C9" s="37"/>
-      <c r="D9" s="37"/>
-      <c r="E9" s="37"/>
-      <c r="F9" s="37"/>
-      <c r="G9" s="37"/>
-      <c r="H9" s="37"/>
-      <c r="I9" s="37"/>
-      <c r="J9" s="38"/>
+      <c r="B9" s="36"/>
+      <c r="C9" s="36"/>
+      <c r="D9" s="36"/>
+      <c r="E9" s="36"/>
+      <c r="F9" s="36"/>
+      <c r="G9" s="36"/>
+      <c r="H9" s="36"/>
+      <c r="I9" s="36"/>
+      <c r="J9" s="37"/>
     </row>
     <row r="10" spans="1:11" ht="29.25">
       <c r="A10" s="2" t="s">
@@ -2375,17 +2381,17 @@
       <c r="B10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="42" t="s">
+      <c r="C10" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="43"/>
+      <c r="D10" s="40"/>
       <c r="E10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="32" t="s">
+      <c r="F10" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="34"/>
+      <c r="G10" s="42"/>
       <c r="H10" s="4" t="s">
         <v>13</v>
       </c>
@@ -2403,15 +2409,15 @@
       <c r="B11" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="23" t="s">
+      <c r="C11" s="51" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="24"/>
+      <c r="D11" s="52"/>
       <c r="E11" s="7"/>
-      <c r="F11" s="21" t="s">
+      <c r="F11" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="25"/>
+      <c r="G11" s="53"/>
       <c r="H11" s="8" t="s">
         <v>16</v>
       </c>
@@ -2421,82 +2427,65 @@
       </c>
     </row>
     <row r="12" spans="1:11" ht="14" customHeight="1">
-      <c r="A12" s="26" t="s">
+      <c r="A12" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="27"/>
-      <c r="C12" s="27"/>
-      <c r="D12" s="27"/>
-      <c r="E12" s="27"/>
-      <c r="F12" s="27"/>
-      <c r="G12" s="27"/>
-      <c r="H12" s="27"/>
-      <c r="I12" s="27"/>
-      <c r="J12" s="28"/>
+      <c r="B12" s="55"/>
+      <c r="C12" s="55"/>
+      <c r="D12" s="55"/>
+      <c r="E12" s="55"/>
+      <c r="F12" s="55"/>
+      <c r="G12" s="55"/>
+      <c r="H12" s="55"/>
+      <c r="I12" s="55"/>
+      <c r="J12" s="56"/>
     </row>
     <row r="13" spans="1:11" ht="14" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="29" t="s">
+      <c r="B13" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="30"/>
-      <c r="D13" s="31"/>
-      <c r="E13" s="32" t="s">
+      <c r="C13" s="58"/>
+      <c r="D13" s="59"/>
+      <c r="E13" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="33"/>
-      <c r="G13" s="34"/>
+      <c r="F13" s="60"/>
+      <c r="G13" s="42"/>
       <c r="H13" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="32" t="s">
+      <c r="I13" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="J13" s="35"/>
+      <c r="J13" s="61"/>
     </row>
     <row r="14" spans="1:11" ht="14" customHeight="1">
       <c r="A14" s="5">
         <v>1</v>
       </c>
-      <c r="B14" s="15" t="s">
+      <c r="B14" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="16"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="18" t="s">
+      <c r="C14" s="44"/>
+      <c r="D14" s="45"/>
+      <c r="E14" s="46" t="s">
         <v>16</v>
       </c>
-      <c r="F14" s="19"/>
-      <c r="G14" s="20"/>
+      <c r="F14" s="47"/>
+      <c r="G14" s="48"/>
       <c r="H14" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="I14" s="21" t="s">
+      <c r="I14" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="J14" s="22"/>
+      <c r="J14" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:J3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="A5:J5"/>
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A7:J7"/>
-    <mergeCell ref="A8:J8"/>
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="F10:G10"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="E14:G14"/>
     <mergeCell ref="I14:J14"/>
@@ -2506,6 +2495,23 @@
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="E13:G13"/>
     <mergeCell ref="I13:J13"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A8:J8"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:J3"/>
   </mergeCells>
   <phoneticPr fontId="30" type="noConversion"/>
   <dataValidations count="2">

</xml_diff>

<commit_message>
更新日报: 2026/09/02 周三 20:30:02.53
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\软通文件\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE137767-E5FF-4459-A9CD-51867629E88C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC2B6581-D1A9-4AFE-82FF-BCF8C2103CCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -483,14 +483,15 @@
   </si>
   <si>
     <t>重点工作: 
-继续做了验收测试指南 包括单点CCAE FusionCare日常巡检 创建主门户 创建策略 以及弹性云服务器申请 注册镜像 以及各种云硬盘操作 以及对象存储服务的测试 
+依照数据治理的文档 学习数据迁移的前置操作 以及需要注意的问题
 重大风险: 无 
 周边求助: 无</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
     <t>重点工作: 
-依照数据治理的文档 学习数据迁移的前置操作 以及需要注意的问题
+继续做了验收测试指南 包括单点CCAE FusionCare日常巡检 创建主门户 创建策略;
+以及弹性云服务器申请 注册镜像 以及各种云硬盘操作 以及对象存储服务的测试;
 重大风险: 无 
 周边求助: 无</t>
     <phoneticPr fontId="30" type="noConversion"/>
@@ -1226,37 +1227,141 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="5" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1283,130 +1388,26 @@
     <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="5" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="166">
@@ -2119,74 +2120,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="22.5" customHeight="1">
-      <c r="A1" s="65" t="s">
+      <c r="A1" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="65"/>
-      <c r="C1" s="65"/>
-      <c r="D1" s="65"/>
-      <c r="E1" s="65"/>
-      <c r="F1" s="65"/>
-      <c r="G1" s="65"/>
-      <c r="H1" s="65"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
     </row>
     <row r="2" spans="1:8" ht="20.25" customHeight="1">
-      <c r="A2" s="66" t="s">
+      <c r="A2" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="67"/>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
     </row>
     <row r="3" spans="1:8" ht="114" customHeight="1">
-      <c r="A3" s="68" t="s">
-        <v>39</v>
-      </c>
-      <c r="B3" s="69"/>
-      <c r="C3" s="69"/>
-      <c r="D3" s="69"/>
-      <c r="E3" s="69"/>
-      <c r="F3" s="69"/>
-      <c r="G3" s="69"/>
-      <c r="H3" s="70"/>
+      <c r="A3" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="B3" s="22"/>
+      <c r="C3" s="22"/>
+      <c r="D3" s="22"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="22"/>
+      <c r="G3" s="22"/>
+      <c r="H3" s="23"/>
     </row>
     <row r="4" spans="1:8" ht="54.75" customHeight="1">
-      <c r="A4" s="66" t="s">
+      <c r="A4" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="67"/>
-      <c r="C4" s="67"/>
-      <c r="D4" s="67"/>
-      <c r="E4" s="67"/>
-      <c r="F4" s="67"/>
-      <c r="G4" s="67"/>
-      <c r="H4" s="67"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="20"/>
+      <c r="H4" s="20"/>
     </row>
     <row r="5" spans="1:8" ht="90" customHeight="1">
-      <c r="A5" s="71" t="s">
-        <v>40</v>
-      </c>
-      <c r="B5" s="72"/>
-      <c r="C5" s="72"/>
-      <c r="D5" s="72"/>
-      <c r="E5" s="72"/>
-      <c r="F5" s="72"/>
-      <c r="G5" s="72"/>
-      <c r="H5" s="73"/>
+      <c r="A5" s="24" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="25"/>
+      <c r="C5" s="25"/>
+      <c r="D5" s="25"/>
+      <c r="E5" s="25"/>
+      <c r="F5" s="25"/>
+      <c r="G5" s="25"/>
+      <c r="H5" s="26"/>
     </row>
     <row r="6" spans="1:8" ht="14.25" customHeight="1">
-      <c r="A6" s="62"/>
-      <c r="B6" s="63"/>
-      <c r="C6" s="63"/>
-      <c r="D6" s="63"/>
-      <c r="E6" s="63"/>
-      <c r="F6" s="63"/>
-      <c r="G6" s="63"/>
-      <c r="H6" s="64"/>
+      <c r="A6" s="15"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2225,154 +2226,154 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.75">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="17"/>
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
+      <c r="D1" s="68"/>
+      <c r="E1" s="68"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="68"/>
+      <c r="H1" s="68"/>
+      <c r="I1" s="68"/>
+      <c r="J1" s="69"/>
     </row>
     <row r="2" spans="1:11" ht="35" customHeight="1">
       <c r="A2" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="58" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="19"/>
+      <c r="C2" s="59"/>
       <c r="D2" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="58" t="s">
         <v>32</v>
       </c>
-      <c r="F2" s="19"/>
+      <c r="F2" s="59"/>
       <c r="G2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="19" t="s">
+      <c r="H2" s="59" t="s">
         <v>36</v>
       </c>
-      <c r="I2" s="19"/>
-      <c r="J2" s="20"/>
+      <c r="I2" s="59"/>
+      <c r="J2" s="70"/>
       <c r="K2" s="9"/>
     </row>
     <row r="3" spans="1:11" ht="15.75">
       <c r="A3" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="58" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="21" t="s">
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="57" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="21"/>
-      <c r="H3" s="22" t="s">
+      <c r="G3" s="57"/>
+      <c r="H3" s="71" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="23"/>
-      <c r="J3" s="24"/>
+      <c r="I3" s="72"/>
+      <c r="J3" s="73"/>
     </row>
     <row r="4" spans="1:11" ht="15.75">
-      <c r="A4" s="25" t="s">
+      <c r="A4" s="56" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="18" t="s">
+      <c r="B4" s="57"/>
+      <c r="C4" s="57"/>
+      <c r="D4" s="57"/>
+      <c r="E4" s="57"/>
+      <c r="F4" s="58" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="19"/>
-      <c r="H4" s="26" t="s">
+      <c r="G4" s="59"/>
+      <c r="H4" s="60" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="27"/>
-      <c r="J4" s="28"/>
+      <c r="I4" s="61"/>
+      <c r="J4" s="62"/>
     </row>
     <row r="5" spans="1:11" ht="20.25">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="63" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="30"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="31"/>
+      <c r="B5" s="64"/>
+      <c r="C5" s="64"/>
+      <c r="D5" s="64"/>
+      <c r="E5" s="64"/>
+      <c r="F5" s="64"/>
+      <c r="G5" s="64"/>
+      <c r="H5" s="64"/>
+      <c r="I5" s="64"/>
+      <c r="J5" s="65"/>
     </row>
     <row r="6" spans="1:11" ht="353" customHeight="1">
-      <c r="A6" s="32" t="s">
+      <c r="A6" s="66" t="s">
         <v>38</v>
       </c>
-      <c r="B6" s="33"/>
-      <c r="C6" s="33"/>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
-      <c r="F6" s="33"/>
-      <c r="G6" s="33"/>
-      <c r="H6" s="33"/>
-      <c r="I6" s="33"/>
-      <c r="J6" s="34"/>
+      <c r="B6" s="52"/>
+      <c r="C6" s="52"/>
+      <c r="D6" s="52"/>
+      <c r="E6" s="52"/>
+      <c r="F6" s="52"/>
+      <c r="G6" s="52"/>
+      <c r="H6" s="52"/>
+      <c r="I6" s="52"/>
+      <c r="J6" s="53"/>
       <c r="K6" s="14" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="20.25">
-      <c r="A7" s="35" t="s">
+      <c r="A7" s="48" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="36"/>
-      <c r="C7" s="36"/>
-      <c r="D7" s="36"/>
-      <c r="E7" s="36"/>
-      <c r="F7" s="36"/>
-      <c r="G7" s="36"/>
-      <c r="H7" s="36"/>
-      <c r="I7" s="36"/>
-      <c r="J7" s="37"/>
+      <c r="B7" s="49"/>
+      <c r="C7" s="49"/>
+      <c r="D7" s="49"/>
+      <c r="E7" s="49"/>
+      <c r="F7" s="49"/>
+      <c r="G7" s="49"/>
+      <c r="H7" s="49"/>
+      <c r="I7" s="49"/>
+      <c r="J7" s="50"/>
     </row>
     <row r="8" spans="1:11" ht="32" customHeight="1">
-      <c r="A8" s="38" t="s">
+      <c r="A8" s="51" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="33"/>
-      <c r="C8" s="33"/>
-      <c r="D8" s="33"/>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="33"/>
-      <c r="I8" s="33"/>
-      <c r="J8" s="34"/>
+      <c r="B8" s="52"/>
+      <c r="C8" s="52"/>
+      <c r="D8" s="52"/>
+      <c r="E8" s="52"/>
+      <c r="F8" s="52"/>
+      <c r="G8" s="52"/>
+      <c r="H8" s="52"/>
+      <c r="I8" s="52"/>
+      <c r="J8" s="53"/>
     </row>
     <row r="9" spans="1:11" ht="20.25">
-      <c r="A9" s="35" t="s">
+      <c r="A9" s="48" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="36"/>
-      <c r="C9" s="36"/>
-      <c r="D9" s="36"/>
-      <c r="E9" s="36"/>
-      <c r="F9" s="36"/>
-      <c r="G9" s="36"/>
-      <c r="H9" s="36"/>
-      <c r="I9" s="36"/>
-      <c r="J9" s="37"/>
+      <c r="B9" s="49"/>
+      <c r="C9" s="49"/>
+      <c r="D9" s="49"/>
+      <c r="E9" s="49"/>
+      <c r="F9" s="49"/>
+      <c r="G9" s="49"/>
+      <c r="H9" s="49"/>
+      <c r="I9" s="49"/>
+      <c r="J9" s="50"/>
     </row>
     <row r="10" spans="1:11" ht="29.25">
       <c r="A10" s="2" t="s">
@@ -2381,17 +2382,17 @@
       <c r="B10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="39" t="s">
+      <c r="C10" s="54" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="40"/>
+      <c r="D10" s="55"/>
       <c r="E10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="41" t="s">
+      <c r="F10" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="42"/>
+      <c r="G10" s="46"/>
       <c r="H10" s="4" t="s">
         <v>13</v>
       </c>
@@ -2409,15 +2410,15 @@
       <c r="B11" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="51" t="s">
+      <c r="C11" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="52"/>
+      <c r="D11" s="36"/>
       <c r="E11" s="7"/>
-      <c r="F11" s="49" t="s">
+      <c r="F11" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="53"/>
+      <c r="G11" s="37"/>
       <c r="H11" s="8" t="s">
         <v>16</v>
       </c>
@@ -2427,65 +2428,82 @@
       </c>
     </row>
     <row r="12" spans="1:11" ht="14" customHeight="1">
-      <c r="A12" s="54" t="s">
+      <c r="A12" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="55"/>
-      <c r="C12" s="55"/>
-      <c r="D12" s="55"/>
-      <c r="E12" s="55"/>
-      <c r="F12" s="55"/>
-      <c r="G12" s="55"/>
-      <c r="H12" s="55"/>
-      <c r="I12" s="55"/>
-      <c r="J12" s="56"/>
+      <c r="B12" s="39"/>
+      <c r="C12" s="39"/>
+      <c r="D12" s="39"/>
+      <c r="E12" s="39"/>
+      <c r="F12" s="39"/>
+      <c r="G12" s="39"/>
+      <c r="H12" s="39"/>
+      <c r="I12" s="39"/>
+      <c r="J12" s="40"/>
     </row>
     <row r="13" spans="1:11" ht="14" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="57" t="s">
+      <c r="B13" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="58"/>
-      <c r="D13" s="59"/>
-      <c r="E13" s="41" t="s">
+      <c r="C13" s="42"/>
+      <c r="D13" s="43"/>
+      <c r="E13" s="44" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="60"/>
-      <c r="G13" s="42"/>
+      <c r="F13" s="45"/>
+      <c r="G13" s="46"/>
       <c r="H13" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="41" t="s">
+      <c r="I13" s="44" t="s">
         <v>21</v>
       </c>
-      <c r="J13" s="61"/>
+      <c r="J13" s="47"/>
     </row>
     <row r="14" spans="1:11" ht="14" customHeight="1">
       <c r="A14" s="5">
         <v>1</v>
       </c>
-      <c r="B14" s="43" t="s">
+      <c r="B14" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="44"/>
-      <c r="D14" s="45"/>
-      <c r="E14" s="46" t="s">
+      <c r="C14" s="28"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="F14" s="47"/>
-      <c r="G14" s="48"/>
+      <c r="F14" s="31"/>
+      <c r="G14" s="32"/>
       <c r="H14" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="I14" s="49" t="s">
+      <c r="I14" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="J14" s="50"/>
+      <c r="J14" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A8:J8"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="F10:G10"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="E14:G14"/>
     <mergeCell ref="I14:J14"/>
@@ -2495,23 +2513,6 @@
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="E13:G13"/>
     <mergeCell ref="I13:J13"/>
-    <mergeCell ref="A7:J7"/>
-    <mergeCell ref="A8:J8"/>
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="A5:J5"/>
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:J3"/>
   </mergeCells>
   <phoneticPr fontId="30" type="noConversion"/>
   <dataValidations count="2">

</xml_diff>

<commit_message>
更新日报: 2026/09/03 周四 17:11:25.47
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\软通文件\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC2B6581-D1A9-4AFE-82FF-BCF8C2103CCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63C078F1-7505-49E4-BCBF-99F9BB7237E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1.日工作简报" sheetId="11" r:id="rId1"/>
@@ -464,7 +464,23 @@
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
-    <t>工作&amp;学习日报-9月2日</t>
+    <t>工作&amp;学习日报-9月3日</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
+    <t>重点工作: 
+学习数据迁移过程 首先迁移DGC的脚本 配置和作业等内容
+然后使用DGC这个迁移工具 批量迁移MRS和DWS的数据
+重大风险: 无 
+周边求助: 无</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
+    <t>重点工作: 
+学习在迁移DGC里的作业 配置和脚本的时候 需要注意什么
+以及迁移过来后需要修改哪些信息才能跑数据迁移
+重大风险: 无 
+周边求助: 无</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
@@ -476,24 +492,9 @@
 周三:
 1. 继续做了验收测试指南 包括单点CCAE FusionCare日常巡检 创建主门户 创建策略 以及弹性云服务器申请 注册镜像 以及各种云硬盘操作 以及对象存储服务的测试
 周四:
-1. 学习了华为云中租户 VDC和企业项目的概念与联系: 其中租户是最高登记的实体用户 创建租户时候 会绑定创建一个一级VDC 然后在创建二级 三级等下级VDC 一级VDC掌握这管理源分配的给他的资源 可以分配给下级VDC 最后在将不同的业务系统对应的虚拟机 划分到不同的企业项目中 实现隔离
+1. 学习数据迁移过程 首先迁移DGC的脚本 配置和作业等内容然后使用DGC这个迁移工具 批量迁移MRS和DWS的数据
 周五:
 1. 学习了客户释放租户过程中 资源释放的过程和规则 1. 清空计算与存储资源 2. 拆除网络拓扑和释放弹性公网ip 3. 解绑资源池并回收资源授权 4. 按层级注销组织实体</t>
-    <phoneticPr fontId="30" type="noConversion"/>
-  </si>
-  <si>
-    <t>重点工作: 
-依照数据治理的文档 学习数据迁移的前置操作 以及需要注意的问题
-重大风险: 无 
-周边求助: 无</t>
-    <phoneticPr fontId="30" type="noConversion"/>
-  </si>
-  <si>
-    <t>重点工作: 
-继续做了验收测试指南 包括单点CCAE FusionCare日常巡检 创建主门户 创建策略;
-以及弹性云服务器申请 注册镜像 以及各种云硬盘操作 以及对象存储服务的测试;
-重大风险: 无 
-周边求助: 无</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
 </sst>
@@ -1263,6 +1264,93 @@
     <xf numFmtId="0" fontId="15" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1316,97 +1404,10 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2145,7 +2146,7 @@
     </row>
     <row r="3" spans="1:8" ht="114" customHeight="1">
       <c r="A3" s="21" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B3" s="22"/>
       <c r="C3" s="22"/>
@@ -2226,154 +2227,154 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.75">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="68"/>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
-      <c r="F1" s="68"/>
-      <c r="G1" s="68"/>
-      <c r="H1" s="68"/>
-      <c r="I1" s="68"/>
-      <c r="J1" s="69"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="29"/>
     </row>
     <row r="2" spans="1:11" ht="35" customHeight="1">
       <c r="A2" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="58" t="s">
+      <c r="B2" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="59"/>
+      <c r="C2" s="31"/>
       <c r="D2" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="E2" s="58" t="s">
+      <c r="E2" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="F2" s="59"/>
+      <c r="F2" s="31"/>
       <c r="G2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="59" t="s">
+      <c r="H2" s="31" t="s">
         <v>36</v>
       </c>
-      <c r="I2" s="59"/>
-      <c r="J2" s="70"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="32"/>
       <c r="K2" s="9"/>
     </row>
     <row r="3" spans="1:11" ht="15.75">
       <c r="A3" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="58" t="s">
+      <c r="B3" s="30" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="57" t="s">
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="57"/>
-      <c r="H3" s="71" t="s">
+      <c r="G3" s="33"/>
+      <c r="H3" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="72"/>
-      <c r="J3" s="73"/>
+      <c r="I3" s="35"/>
+      <c r="J3" s="36"/>
     </row>
     <row r="4" spans="1:11" ht="15.75">
-      <c r="A4" s="56" t="s">
+      <c r="A4" s="37" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="57"/>
-      <c r="C4" s="57"/>
-      <c r="D4" s="57"/>
-      <c r="E4" s="57"/>
-      <c r="F4" s="58" t="s">
+      <c r="B4" s="33"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
+      <c r="F4" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="59"/>
-      <c r="H4" s="60" t="s">
+      <c r="G4" s="31"/>
+      <c r="H4" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="61"/>
-      <c r="J4" s="62"/>
+      <c r="I4" s="39"/>
+      <c r="J4" s="40"/>
     </row>
     <row r="5" spans="1:11" ht="20.25">
-      <c r="A5" s="63" t="s">
+      <c r="A5" s="41" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="64"/>
-      <c r="C5" s="64"/>
-      <c r="D5" s="64"/>
-      <c r="E5" s="64"/>
-      <c r="F5" s="64"/>
-      <c r="G5" s="64"/>
-      <c r="H5" s="64"/>
-      <c r="I5" s="64"/>
-      <c r="J5" s="65"/>
+      <c r="B5" s="42"/>
+      <c r="C5" s="42"/>
+      <c r="D5" s="42"/>
+      <c r="E5" s="42"/>
+      <c r="F5" s="42"/>
+      <c r="G5" s="42"/>
+      <c r="H5" s="42"/>
+      <c r="I5" s="42"/>
+      <c r="J5" s="43"/>
     </row>
     <row r="6" spans="1:11" ht="353" customHeight="1">
-      <c r="A6" s="66" t="s">
-        <v>38</v>
-      </c>
-      <c r="B6" s="52"/>
-      <c r="C6" s="52"/>
-      <c r="D6" s="52"/>
-      <c r="E6" s="52"/>
-      <c r="F6" s="52"/>
-      <c r="G6" s="52"/>
-      <c r="H6" s="52"/>
-      <c r="I6" s="52"/>
-      <c r="J6" s="53"/>
+      <c r="A6" s="44" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="45"/>
+      <c r="C6" s="45"/>
+      <c r="D6" s="45"/>
+      <c r="E6" s="45"/>
+      <c r="F6" s="45"/>
+      <c r="G6" s="45"/>
+      <c r="H6" s="45"/>
+      <c r="I6" s="45"/>
+      <c r="J6" s="46"/>
       <c r="K6" s="14" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="20.25">
-      <c r="A7" s="48" t="s">
+      <c r="A7" s="47" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="49"/>
-      <c r="C7" s="49"/>
-      <c r="D7" s="49"/>
-      <c r="E7" s="49"/>
-      <c r="F7" s="49"/>
-      <c r="G7" s="49"/>
-      <c r="H7" s="49"/>
-      <c r="I7" s="49"/>
-      <c r="J7" s="50"/>
+      <c r="B7" s="48"/>
+      <c r="C7" s="48"/>
+      <c r="D7" s="48"/>
+      <c r="E7" s="48"/>
+      <c r="F7" s="48"/>
+      <c r="G7" s="48"/>
+      <c r="H7" s="48"/>
+      <c r="I7" s="48"/>
+      <c r="J7" s="49"/>
     </row>
     <row r="8" spans="1:11" ht="32" customHeight="1">
-      <c r="A8" s="51" t="s">
+      <c r="A8" s="50" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="52"/>
-      <c r="C8" s="52"/>
-      <c r="D8" s="52"/>
-      <c r="E8" s="52"/>
-      <c r="F8" s="52"/>
-      <c r="G8" s="52"/>
-      <c r="H8" s="52"/>
-      <c r="I8" s="52"/>
-      <c r="J8" s="53"/>
+      <c r="B8" s="45"/>
+      <c r="C8" s="45"/>
+      <c r="D8" s="45"/>
+      <c r="E8" s="45"/>
+      <c r="F8" s="45"/>
+      <c r="G8" s="45"/>
+      <c r="H8" s="45"/>
+      <c r="I8" s="45"/>
+      <c r="J8" s="46"/>
     </row>
     <row r="9" spans="1:11" ht="20.25">
-      <c r="A9" s="48" t="s">
+      <c r="A9" s="47" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="49"/>
-      <c r="C9" s="49"/>
-      <c r="D9" s="49"/>
-      <c r="E9" s="49"/>
-      <c r="F9" s="49"/>
-      <c r="G9" s="49"/>
-      <c r="H9" s="49"/>
-      <c r="I9" s="49"/>
-      <c r="J9" s="50"/>
+      <c r="B9" s="48"/>
+      <c r="C9" s="48"/>
+      <c r="D9" s="48"/>
+      <c r="E9" s="48"/>
+      <c r="F9" s="48"/>
+      <c r="G9" s="48"/>
+      <c r="H9" s="48"/>
+      <c r="I9" s="48"/>
+      <c r="J9" s="49"/>
     </row>
     <row r="10" spans="1:11" ht="29.25">
       <c r="A10" s="2" t="s">
@@ -2382,17 +2383,17 @@
       <c r="B10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="54" t="s">
+      <c r="C10" s="51" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="55"/>
+      <c r="D10" s="52"/>
       <c r="E10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="44" t="s">
+      <c r="F10" s="53" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="46"/>
+      <c r="G10" s="54"/>
       <c r="H10" s="4" t="s">
         <v>13</v>
       </c>
@@ -2410,15 +2411,15 @@
       <c r="B11" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="35" t="s">
+      <c r="C11" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="36"/>
+      <c r="D11" s="64"/>
       <c r="E11" s="7"/>
-      <c r="F11" s="33" t="s">
+      <c r="F11" s="61" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="37"/>
+      <c r="G11" s="65"/>
       <c r="H11" s="8" t="s">
         <v>16</v>
       </c>
@@ -2428,82 +2429,65 @@
       </c>
     </row>
     <row r="12" spans="1:11" ht="14" customHeight="1">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="66" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="39"/>
-      <c r="C12" s="39"/>
-      <c r="D12" s="39"/>
-      <c r="E12" s="39"/>
-      <c r="F12" s="39"/>
-      <c r="G12" s="39"/>
-      <c r="H12" s="39"/>
-      <c r="I12" s="39"/>
-      <c r="J12" s="40"/>
+      <c r="B12" s="67"/>
+      <c r="C12" s="67"/>
+      <c r="D12" s="67"/>
+      <c r="E12" s="67"/>
+      <c r="F12" s="67"/>
+      <c r="G12" s="67"/>
+      <c r="H12" s="67"/>
+      <c r="I12" s="67"/>
+      <c r="J12" s="68"/>
     </row>
     <row r="13" spans="1:11" ht="14" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="41" t="s">
+      <c r="B13" s="69" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="42"/>
-      <c r="D13" s="43"/>
-      <c r="E13" s="44" t="s">
+      <c r="C13" s="70"/>
+      <c r="D13" s="71"/>
+      <c r="E13" s="53" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="45"/>
-      <c r="G13" s="46"/>
+      <c r="F13" s="72"/>
+      <c r="G13" s="54"/>
       <c r="H13" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="44" t="s">
+      <c r="I13" s="53" t="s">
         <v>21</v>
       </c>
-      <c r="J13" s="47"/>
+      <c r="J13" s="73"/>
     </row>
     <row r="14" spans="1:11" ht="14" customHeight="1">
       <c r="A14" s="5">
         <v>1</v>
       </c>
-      <c r="B14" s="27" t="s">
+      <c r="B14" s="55" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="28"/>
-      <c r="D14" s="29"/>
-      <c r="E14" s="30" t="s">
+      <c r="C14" s="56"/>
+      <c r="D14" s="57"/>
+      <c r="E14" s="58" t="s">
         <v>16</v>
       </c>
-      <c r="F14" s="31"/>
-      <c r="G14" s="32"/>
+      <c r="F14" s="59"/>
+      <c r="G14" s="60"/>
       <c r="H14" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="I14" s="33" t="s">
+      <c r="I14" s="61" t="s">
         <v>16</v>
       </c>
-      <c r="J14" s="34"/>
+      <c r="J14" s="62"/>
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:J3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="A5:J5"/>
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A7:J7"/>
-    <mergeCell ref="A8:J8"/>
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="F10:G10"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="E14:G14"/>
     <mergeCell ref="I14:J14"/>
@@ -2513,6 +2497,23 @@
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="E13:G13"/>
     <mergeCell ref="I13:J13"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A8:J8"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:J3"/>
   </mergeCells>
   <phoneticPr fontId="30" type="noConversion"/>
   <dataValidations count="2">

</xml_diff>

<commit_message>
更新日报: 2026/09/04 周五 16:04:36.04
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\软通文件\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63C078F1-7505-49E4-BCBF-99F9BB7237E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99FC725A-2F14-49DE-B4F8-5E6826124926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -464,23 +464,22 @@
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
-    <t>工作&amp;学习日报-9月3日</t>
-    <phoneticPr fontId="30" type="noConversion"/>
-  </si>
-  <si>
     <t>重点工作: 
-学习数据迁移过程 首先迁移DGC的脚本 配置和作业等内容
-然后使用DGC这个迁移工具 批量迁移MRS和DWS的数据
+1. 学习了DataArts Studio资源迁移的全过程 以及约束条件 迁移选择的工具等
+2. 学习DataArts Studio支持的数据源包括哪些 以及连接参数怎么写
 重大风险: 无 
 周边求助: 无</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
     <t>重点工作: 
-学习在迁移DGC里的作业 配置和脚本的时候 需要注意什么
-以及迁移过来后需要修改哪些信息才能跑数据迁移
+学习数据集成CDM如何离线作业
 重大风险: 无 
 周边求助: 无</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
+    <t>工作&amp;学习日报-9月4日</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
@@ -494,7 +493,8 @@
 周四:
 1. 学习数据迁移过程 首先迁移DGC的脚本 配置和作业等内容然后使用DGC这个迁移工具 批量迁移MRS和DWS的数据
 周五:
-1. 学习了客户释放租户过程中 资源释放的过程和规则 1. 清空计算与存储资源 2. 拆除网络拓扑和释放弹性公网ip 3. 解绑资源池并回收资源授权 4. 按层级注销组织实体</t>
+1. 学习了DataArts Studio资源迁移的全过程 以及约束条件 迁移选择的工具等 使用OBS桶或者将作业 配置和脚本等压缩成zip文件导出到本地 然后在新的工作空间导入
+2. 学习DataArts Studio支持的数据源包括哪些 以及连接参数怎么写</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
 </sst>
@@ -1228,6 +1228,152 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="5" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1263,152 +1409,6 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="5" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="166">
@@ -2121,74 +2121,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="22.5" customHeight="1">
-      <c r="A1" s="18" t="s">
-        <v>37</v>
-      </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
+      <c r="A1" s="65" t="s">
+        <v>39</v>
+      </c>
+      <c r="B1" s="65"/>
+      <c r="C1" s="65"/>
+      <c r="D1" s="65"/>
+      <c r="E1" s="65"/>
+      <c r="F1" s="65"/>
+      <c r="G1" s="65"/>
+      <c r="H1" s="65"/>
     </row>
     <row r="2" spans="1:8" ht="20.25" customHeight="1">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="66" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
+      <c r="B2" s="67"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
     </row>
     <row r="3" spans="1:8" ht="114" customHeight="1">
-      <c r="A3" s="21" t="s">
-        <v>38</v>
-      </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="23"/>
+      <c r="A3" s="68" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="69"/>
+      <c r="C3" s="69"/>
+      <c r="D3" s="69"/>
+      <c r="E3" s="69"/>
+      <c r="F3" s="69"/>
+      <c r="G3" s="69"/>
+      <c r="H3" s="70"/>
     </row>
     <row r="4" spans="1:8" ht="54.75" customHeight="1">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="66" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="20"/>
-      <c r="H4" s="20"/>
+      <c r="B4" s="67"/>
+      <c r="C4" s="67"/>
+      <c r="D4" s="67"/>
+      <c r="E4" s="67"/>
+      <c r="F4" s="67"/>
+      <c r="G4" s="67"/>
+      <c r="H4" s="67"/>
     </row>
     <row r="5" spans="1:8" ht="90" customHeight="1">
-      <c r="A5" s="24" t="s">
-        <v>39</v>
-      </c>
-      <c r="B5" s="25"/>
-      <c r="C5" s="25"/>
-      <c r="D5" s="25"/>
-      <c r="E5" s="25"/>
-      <c r="F5" s="25"/>
-      <c r="G5" s="25"/>
-      <c r="H5" s="26"/>
+      <c r="A5" s="71" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" s="72"/>
+      <c r="C5" s="72"/>
+      <c r="D5" s="72"/>
+      <c r="E5" s="72"/>
+      <c r="F5" s="72"/>
+      <c r="G5" s="72"/>
+      <c r="H5" s="73"/>
     </row>
     <row r="6" spans="1:8" ht="14.25" customHeight="1">
-      <c r="A6" s="15"/>
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="16"/>
-      <c r="H6" s="17"/>
+      <c r="A6" s="62"/>
+      <c r="B6" s="63"/>
+      <c r="C6" s="63"/>
+      <c r="D6" s="63"/>
+      <c r="E6" s="63"/>
+      <c r="F6" s="63"/>
+      <c r="G6" s="63"/>
+      <c r="H6" s="64"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2227,154 +2227,154 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.75">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="55" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
-      <c r="I1" s="28"/>
-      <c r="J1" s="29"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="57"/>
     </row>
     <row r="2" spans="1:11" ht="35" customHeight="1">
       <c r="A2" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="46" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="31"/>
+      <c r="C2" s="47"/>
       <c r="D2" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="E2" s="30" t="s">
+      <c r="E2" s="46" t="s">
         <v>32</v>
       </c>
-      <c r="F2" s="31"/>
+      <c r="F2" s="47"/>
       <c r="G2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="31" t="s">
+      <c r="H2" s="47" t="s">
         <v>36</v>
       </c>
-      <c r="I2" s="31"/>
-      <c r="J2" s="32"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="58"/>
       <c r="K2" s="9"/>
     </row>
     <row r="3" spans="1:11" ht="15.75">
       <c r="A3" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="46" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="33" t="s">
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="33"/>
-      <c r="H3" s="34" t="s">
+      <c r="G3" s="45"/>
+      <c r="H3" s="59" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="35"/>
-      <c r="J3" s="36"/>
+      <c r="I3" s="60"/>
+      <c r="J3" s="61"/>
     </row>
     <row r="4" spans="1:11" ht="15.75">
-      <c r="A4" s="37" t="s">
+      <c r="A4" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="33"/>
-      <c r="C4" s="33"/>
-      <c r="D4" s="33"/>
-      <c r="E4" s="33"/>
-      <c r="F4" s="30" t="s">
+      <c r="B4" s="45"/>
+      <c r="C4" s="45"/>
+      <c r="D4" s="45"/>
+      <c r="E4" s="45"/>
+      <c r="F4" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="31"/>
-      <c r="H4" s="38" t="s">
+      <c r="G4" s="47"/>
+      <c r="H4" s="48" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="39"/>
-      <c r="J4" s="40"/>
+      <c r="I4" s="49"/>
+      <c r="J4" s="50"/>
     </row>
     <row r="5" spans="1:11" ht="20.25">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="42"/>
-      <c r="C5" s="42"/>
-      <c r="D5" s="42"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="42"/>
-      <c r="I5" s="42"/>
-      <c r="J5" s="43"/>
+      <c r="B5" s="52"/>
+      <c r="C5" s="52"/>
+      <c r="D5" s="52"/>
+      <c r="E5" s="52"/>
+      <c r="F5" s="52"/>
+      <c r="G5" s="52"/>
+      <c r="H5" s="52"/>
+      <c r="I5" s="52"/>
+      <c r="J5" s="53"/>
     </row>
     <row r="6" spans="1:11" ht="353" customHeight="1">
-      <c r="A6" s="44" t="s">
+      <c r="A6" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="45"/>
-      <c r="C6" s="45"/>
-      <c r="D6" s="45"/>
-      <c r="E6" s="45"/>
-      <c r="F6" s="45"/>
-      <c r="G6" s="45"/>
-      <c r="H6" s="45"/>
-      <c r="I6" s="45"/>
-      <c r="J6" s="46"/>
+      <c r="B6" s="40"/>
+      <c r="C6" s="40"/>
+      <c r="D6" s="40"/>
+      <c r="E6" s="40"/>
+      <c r="F6" s="40"/>
+      <c r="G6" s="40"/>
+      <c r="H6" s="40"/>
+      <c r="I6" s="40"/>
+      <c r="J6" s="41"/>
       <c r="K6" s="14" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="20.25">
-      <c r="A7" s="47" t="s">
+      <c r="A7" s="36" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="48"/>
-      <c r="C7" s="48"/>
-      <c r="D7" s="48"/>
-      <c r="E7" s="48"/>
-      <c r="F7" s="48"/>
-      <c r="G7" s="48"/>
-      <c r="H7" s="48"/>
-      <c r="I7" s="48"/>
-      <c r="J7" s="49"/>
+      <c r="B7" s="37"/>
+      <c r="C7" s="37"/>
+      <c r="D7" s="37"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="37"/>
+      <c r="I7" s="37"/>
+      <c r="J7" s="38"/>
     </row>
     <row r="8" spans="1:11" ht="32" customHeight="1">
-      <c r="A8" s="50" t="s">
+      <c r="A8" s="39" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="45"/>
-      <c r="C8" s="45"/>
-      <c r="D8" s="45"/>
-      <c r="E8" s="45"/>
-      <c r="F8" s="45"/>
-      <c r="G8" s="45"/>
-      <c r="H8" s="45"/>
-      <c r="I8" s="45"/>
-      <c r="J8" s="46"/>
+      <c r="B8" s="40"/>
+      <c r="C8" s="40"/>
+      <c r="D8" s="40"/>
+      <c r="E8" s="40"/>
+      <c r="F8" s="40"/>
+      <c r="G8" s="40"/>
+      <c r="H8" s="40"/>
+      <c r="I8" s="40"/>
+      <c r="J8" s="41"/>
     </row>
     <row r="9" spans="1:11" ht="20.25">
-      <c r="A9" s="47" t="s">
+      <c r="A9" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="48"/>
-      <c r="C9" s="48"/>
-      <c r="D9" s="48"/>
-      <c r="E9" s="48"/>
-      <c r="F9" s="48"/>
-      <c r="G9" s="48"/>
-      <c r="H9" s="48"/>
-      <c r="I9" s="48"/>
-      <c r="J9" s="49"/>
+      <c r="B9" s="37"/>
+      <c r="C9" s="37"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="37"/>
+      <c r="F9" s="37"/>
+      <c r="G9" s="37"/>
+      <c r="H9" s="37"/>
+      <c r="I9" s="37"/>
+      <c r="J9" s="38"/>
     </row>
     <row r="10" spans="1:11" ht="29.25">
       <c r="A10" s="2" t="s">
@@ -2383,17 +2383,17 @@
       <c r="B10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="51" t="s">
+      <c r="C10" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="52"/>
+      <c r="D10" s="43"/>
       <c r="E10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="53" t="s">
+      <c r="F10" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="54"/>
+      <c r="G10" s="34"/>
       <c r="H10" s="4" t="s">
         <v>13</v>
       </c>
@@ -2411,15 +2411,15 @@
       <c r="B11" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="63" t="s">
+      <c r="C11" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="64"/>
+      <c r="D11" s="24"/>
       <c r="E11" s="7"/>
-      <c r="F11" s="61" t="s">
+      <c r="F11" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="65"/>
+      <c r="G11" s="25"/>
       <c r="H11" s="8" t="s">
         <v>16</v>
       </c>
@@ -2429,65 +2429,82 @@
       </c>
     </row>
     <row r="12" spans="1:11" ht="14" customHeight="1">
-      <c r="A12" s="66" t="s">
+      <c r="A12" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="67"/>
-      <c r="C12" s="67"/>
-      <c r="D12" s="67"/>
-      <c r="E12" s="67"/>
-      <c r="F12" s="67"/>
-      <c r="G12" s="67"/>
-      <c r="H12" s="67"/>
-      <c r="I12" s="67"/>
-      <c r="J12" s="68"/>
+      <c r="B12" s="27"/>
+      <c r="C12" s="27"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="27"/>
+      <c r="F12" s="27"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="27"/>
+      <c r="I12" s="27"/>
+      <c r="J12" s="28"/>
     </row>
     <row r="13" spans="1:11" ht="14" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="69" t="s">
+      <c r="B13" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="70"/>
-      <c r="D13" s="71"/>
-      <c r="E13" s="53" t="s">
+      <c r="C13" s="30"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="72"/>
-      <c r="G13" s="54"/>
+      <c r="F13" s="33"/>
+      <c r="G13" s="34"/>
       <c r="H13" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="53" t="s">
+      <c r="I13" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="J13" s="73"/>
+      <c r="J13" s="35"/>
     </row>
     <row r="14" spans="1:11" ht="14" customHeight="1">
       <c r="A14" s="5">
         <v>1</v>
       </c>
-      <c r="B14" s="55" t="s">
+      <c r="B14" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="56"/>
-      <c r="D14" s="57"/>
-      <c r="E14" s="58" t="s">
+      <c r="C14" s="16"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="F14" s="59"/>
-      <c r="G14" s="60"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="20"/>
       <c r="H14" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="I14" s="61" t="s">
+      <c r="I14" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="J14" s="62"/>
+      <c r="J14" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A8:J8"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="F10:G10"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="E14:G14"/>
     <mergeCell ref="I14:J14"/>
@@ -2497,23 +2514,6 @@
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="E13:G13"/>
     <mergeCell ref="I13:J13"/>
-    <mergeCell ref="A7:J7"/>
-    <mergeCell ref="A8:J8"/>
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="A5:J5"/>
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:J3"/>
   </mergeCells>
   <phoneticPr fontId="30" type="noConversion"/>
   <dataValidations count="2">

</xml_diff>